<commit_message>
feat: add rapid digital-run liquidity stress scenario
Add a severe exploratory deposit-run scenario with front-loaded outflows, scenario-specific HQLA market-value shocks, a seven-day survival horizon, expanded validation, and refreshed ALCO deliverables.
</commit_message>
<xml_diff>
--- a/excel/Aurelia_Bank_ALCO_Risk_Workbench.xlsx
+++ b/excel/Aurelia_Bank_ALCO_Risk_Workbench.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="R7ca96f742fc34f50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R74d0fc161a134b02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="3" r:id="Re6c1f541f9a14706"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions Raw" sheetId="4" r:id="R11cb1113276b4f36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repricing Gap" sheetId="5" r:id="R8e08caf6c0174281"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IRRBB EVE" sheetId="6" r:id="R0c8d82c150484465"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NII Sensitivity" sheetId="7" r:id="R39c9b6df87744d80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liquidity" sheetId="8" r:id="Rbabadf0e8ff74114"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Hedge" sheetId="9" r:id="Rf9cf619124b34895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="10" r:id="R941d789cb3d0495e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="11" r:id="R523c953894234e0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="R2646fe77c57746d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R2c001d998e214b0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="3" r:id="R4c5f00fc29a74b55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions Raw" sheetId="4" r:id="Ra028822a1a274df8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repricing Gap" sheetId="5" r:id="Rbff1f6e00c114311"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IRRBB EVE" sheetId="6" r:id="R2f9c3bcd401d4451"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NII Sensitivity" sheetId="7" r:id="Re8498d649e104563"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liquidity" sheetId="8" r:id="R0b21fc60ca81473d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Hedge" sheetId="9" r:id="Rb3ef797d121c4a7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="10" r:id="R11249d17e03e4807"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="11" r:id="Re1f0334f7d5c4880"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,9 +20,9 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={9797CADA-ED84-CD56-90A0-55F03189A0F9}</x:author>
-    <x:author>tc={8B3D5F63-A3BE-10AA-5BD3-D8C17FABF35A}</x:author>
-    <x:author>tc={4A2F2257-0EC2-5C1F-0FC0-38DECE0247FF}</x:author>
+    <x:author>tc={C98EFE8F-088B-9606-9A45-E7FFDB6B4E80}</x:author>
+    <x:author>tc={270A24B8-4951-F9F8-1C31-B4A5E3B1C483}</x:author>
+    <x:author>tc={867C2A4C-7032-EFE8-6FE6-86305A326678}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B6" authorId="0">
@@ -221,7 +221,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="20">
+  <x:borders count="26">
     <x:border/>
     <x:border>
       <x:bottom style="double">
@@ -350,6 +350,48 @@
     </x:border>
     <x:border>
       <x:left style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:left>
+      <x:top style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:right>
+      <x:top style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:left>
+      <x:bottom style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:right>
+      <x:bottom style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="medium">
         <x:color rgb="FFC9D5DF"/>
       </x:left>
       <x:top style="medium">
@@ -394,7 +436,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="144">
+  <x:cellXfs count="162">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -482,6 +524,40 @@
     <x:xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="8" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="206" fontId="8" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="9" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="9" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="9" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="9" fillId="8" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="8" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="201" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -509,140 +585,140 @@
     <x:xf numFmtId="207" fontId="13" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="13" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="8" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="8" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="9" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="9" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="9" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="208" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1061,7 +1137,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>Combined stress takes LCR proxy below 100%</a:t>
+              <a:t>Rapid digital run exposes a seven-day survival horizon</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1080,7 +1156,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Executive Dashboard'!$H$19:$H$22</c:f>
+              <c:f>'Executive Dashboard'!$H$19:$H$23</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1088,7 +1164,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Executive Dashboard'!$I$19:$I$22</c:f>
+              <c:f>'Executive Dashboard'!$I$19:$I$23</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1443,7 +1519,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>LCR proxy under stress scenarios</a:t>
+              <a:t>Rapid digital run drives the LCR proxy to 78.1%</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1462,7 +1538,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Liquidity'!$L$8:$L$11</c:f>
+              <c:f>'Liquidity'!$N$8:$N$12</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1470,7 +1546,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Liquidity'!$M$8:$M$11</c:f>
+              <c:f>'Liquidity'!$O$8:$O$12</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1569,7 +1645,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R43ab1af045894983"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R366b5dbf276a4ca5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1599,7 +1675,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5c7b3c86ecce4fe7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R94bdfbe0b7ce4d2e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1634,7 +1710,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R05fd5df7c001460a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc7d492c98aeb41a2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1669,7 +1745,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0e213e15d56144dc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f91b34600324792"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1688,7 +1764,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1704,7 +1780,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R76806bd2dc7d4c13"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9ff97a2fcaf64970"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1715,7 +1791,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Murat Miraç Gedik" id="{A6D395B8-2D65-416B-B4C7-A973252CAC41}"/>
+  <xltc:person displayName="Murat Miraç Gedik" id="{6A530232-7AB4-4679-A611-99B52FBDEE6F}"/>
 </xltc:personList>
 </file>
 
@@ -1912,13 +1988,13 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B6" dT="2026-08-20T10:13:18.316" personId="{A6D395B8-2D65-416B-B4C7-A973252CAC41}" id="{9797CADA-ED84-CD56-90A0-55F03189A0F9}">
+  <xltc:threadedComment ref="B6" dT="2026-08-21T11:42:35.52" personId="{6A530232-7AB4-4679-A611-99B52FBDEE6F}" id="{C98EFE8F-088B-9606-9A45-E7FFDB6B4E80}">
     <xltc:text>Source: TCMB policy-rate announcement (2026 reference). https://www.tcmb.gov.tr/wps/wcm/connect/tr/tcmb+tr/main+menu/duyurular/basin/2026/duy2026-23</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B7" dT="2026-08-20T10:13:18.316" personId="{A6D395B8-2D65-416B-B4C7-A973252CAC41}" id="{8B3D5F63-A3BE-10AA-5BD3-D8C17FABF35A}">
+  <xltc:threadedComment ref="B7" dT="2026-08-21T11:42:35.52" personId="{6A530232-7AB4-4679-A611-99B52FBDEE6F}" id="{270A24B8-4951-F9F8-1C31-B4A5E3B1C483}">
     <xltc:text>Source: TCMB official exchange rates via e-Devlet, 2026-08-19. https://www.turkiye.gov.tr/doviz-kurlari</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="F6" dT="2026-08-20T10:13:18.316" personId="{A6D395B8-2D65-416B-B4C7-A973252CAC41}" id="{4A2F2257-0EC2-5C1F-0FC0-38DECE0247FF}">
+  <xltc:threadedComment ref="F6" dT="2026-08-21T11:42:35.52" personId="{6A530232-7AB4-4679-A611-99B52FBDEE6F}" id="{867C2A4C-7032-EFE8-6FE6-86305A326678}">
     <xltc:text>Source: Basel Committee, recalibration of IRRBB shocks (d578), effective 2026-01-01. https://www.bis.org/bcbs/publ/d578.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -1989,76 +2065,76 @@
       <x:c r="L3" s="1"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="78" t="str">
+      <x:c r="A4" s="96" t="str">
         <x:v>TOTAL ASSETS</x:v>
       </x:c>
-      <x:c r="B4" s="78"/>
-      <x:c r="C4" s="78" t="str">
+      <x:c r="B4" s="96"/>
+      <x:c r="C4" s="96" t="str">
         <x:v>WORST EVE LOSS</x:v>
       </x:c>
-      <x:c r="D4" s="78"/>
-      <x:c r="E4" s="78" t="str">
+      <x:c r="D4" s="96"/>
+      <x:c r="E4" s="96" t="str">
         <x:v>MAX |DELTA NII|</x:v>
       </x:c>
-      <x:c r="F4" s="78"/>
-      <x:c r="G4" s="78" t="str">
+      <x:c r="F4" s="96"/>
+      <x:c r="G4" s="96" t="str">
         <x:v>COMBINED LCR</x:v>
       </x:c>
-      <x:c r="H4" s="78"/>
-      <x:c r="I4" s="78" t="str">
+      <x:c r="H4" s="96"/>
+      <x:c r="I4" s="96" t="str">
         <x:v>FX OPEN / EQUITY</x:v>
       </x:c>
-      <x:c r="J4" s="78"/>
-      <x:c r="K4" s="78" t="str">
+      <x:c r="J4" s="96"/>
+      <x:c r="K4" s="96" t="str">
         <x:v>MODEL STATUS</x:v>
       </x:c>
-      <x:c r="L4" s="78"/>
+      <x:c r="L4" s="96"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="116" t="n">
+      <x:c r="A5" s="134" t="n">
         <x:f>'Balance Sheet'!F25</x:f>
         <x:v>180000</x:v>
       </x:c>
-      <x:c r="B5" s="117"/>
-      <x:c r="C5" s="126" t="n">
+      <x:c r="B5" s="135"/>
+      <x:c r="C5" s="144" t="n">
         <x:f>'IRRBB EVE'!C4</x:f>
         <x:v>0.13743893711111127</x:v>
       </x:c>
-      <x:c r="D5" s="126"/>
-      <x:c r="E5" s="118" t="n">
+      <x:c r="D5" s="144"/>
+      <x:c r="E5" s="136" t="n">
         <x:f>'NII Sensitivity'!C4</x:f>
         <x:v>0.058133649698356125</x:v>
       </x:c>
-      <x:c r="F5" s="118"/>
-      <x:c r="G5" s="128" t="n">
+      <x:c r="F5" s="136"/>
+      <x:c r="G5" s="146" t="n">
         <x:f>Liquidity!C4</x:f>
         <x:v>0.9483364199501884</x:v>
       </x:c>
-      <x:c r="H5" s="128"/>
-      <x:c r="I5" s="126" t="n">
+      <x:c r="H5" s="146"/>
+      <x:c r="I5" s="144" t="n">
         <x:f>'FX &amp; Hedge'!C4</x:f>
         <x:v>0.3333333333333333</x:v>
       </x:c>
-      <x:c r="J5" s="126"/>
-      <x:c r="K5" s="134" t="str">
+      <x:c r="J5" s="144"/>
+      <x:c r="K5" s="152" t="str">
         <x:f>Controls!F30</x:f>
         <x:v>OK - RISK FLAGS SURFACED</x:v>
       </x:c>
-      <x:c r="L5" s="135"/>
+      <x:c r="L5" s="153"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="121"/>
-      <x:c r="B6" s="122"/>
-      <x:c r="C6" s="127"/>
-      <x:c r="D6" s="127"/>
-      <x:c r="E6" s="123"/>
-      <x:c r="F6" s="123"/>
-      <x:c r="G6" s="129"/>
-      <x:c r="H6" s="129"/>
-      <x:c r="I6" s="127"/>
-      <x:c r="J6" s="127"/>
-      <x:c r="K6" s="136"/>
-      <x:c r="L6" s="137"/>
+      <x:c r="A6" s="139"/>
+      <x:c r="B6" s="140"/>
+      <x:c r="C6" s="145"/>
+      <x:c r="D6" s="145"/>
+      <x:c r="E6" s="141"/>
+      <x:c r="F6" s="141"/>
+      <x:c r="G6" s="147"/>
+      <x:c r="H6" s="147"/>
+      <x:c r="I6" s="145"/>
+      <x:c r="J6" s="145"/>
+      <x:c r="K6" s="154"/>
+      <x:c r="L6" s="155"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1"/>
@@ -2112,23 +2188,23 @@
         <x:v>ALCO interpretation</x:v>
       </x:c>
       <x:c r="G9" s="1"/>
-      <x:c r="H9" s="142" t="str">
+      <x:c r="H9" s="160" t="str">
         <x:v>1 | Approve an 80% FX hedge target: buy USD/EUR and sell TRY via FX swap or forward, subject to limits and execution controls.</x:v>
       </x:c>
-      <x:c r="I9" s="142"/>
-      <x:c r="J9" s="142"/>
-      <x:c r="K9" s="142"/>
-      <x:c r="L9" s="142"/>
+      <x:c r="I9" s="160"/>
+      <x:c r="J9" s="160"/>
+      <x:c r="K9" s="160"/>
+      <x:c r="L9" s="160"/>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="1" t="str">
         <x:v>EVE loss / Tier 1</x:v>
       </x:c>
-      <x:c r="B10" s="69" t="n">
+      <x:c r="B10" s="87" t="n">
         <x:f>'IRRBB EVE'!C4</x:f>
         <x:v>0.13743893711111127</x:v>
       </x:c>
-      <x:c r="C10" s="69" t="n">
+      <x:c r="C10" s="87" t="n">
         <x:f>Assumptions!B11</x:f>
         <x:v>0.15</x:v>
       </x:c>
@@ -2140,27 +2216,27 @@
         <x:f>IF(B10&lt;=C10,"WITHIN_LIMIT","BREACH")</x:f>
         <x:v>WITHIN_LIMIT</x:v>
       </x:c>
-      <x:c r="F10" s="70" t="str">
+      <x:c r="F10" s="88" t="str">
         <x:v>Parallel-up is the adverse EVE scenario</x:v>
       </x:c>
       <x:c r="G10" s="1"/>
-      <x:c r="H10" s="142" t="str">
+      <x:c r="H10" s="160" t="str">
         <x:v>2 | Preserve the liquidity buffer: combined-stress LCR proxy is 94.8% and survival reaches the 30-day floor.</x:v>
       </x:c>
-      <x:c r="I10" s="142"/>
-      <x:c r="J10" s="142"/>
-      <x:c r="K10" s="142"/>
-      <x:c r="L10" s="142"/>
+      <x:c r="I10" s="160"/>
+      <x:c r="J10" s="160"/>
+      <x:c r="K10" s="160"/>
+      <x:c r="L10" s="160"/>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
       <x:c r="A11" s="1" t="str">
         <x:v>Absolute Delta NII</x:v>
       </x:c>
-      <x:c r="B11" s="69" t="n">
+      <x:c r="B11" s="87" t="n">
         <x:f>'NII Sensitivity'!C4</x:f>
         <x:v>0.058133649698356125</x:v>
       </x:c>
-      <x:c r="C11" s="69" t="n">
+      <x:c r="C11" s="87" t="n">
         <x:f>Assumptions!B12</x:f>
         <x:v>0.12</x:v>
       </x:c>
@@ -2172,27 +2248,27 @@
         <x:f>IF(B11&lt;=C11,"WITHIN_LIMIT","BREACH")</x:f>
         <x:v>WITHIN_LIMIT</x:v>
       </x:c>
-      <x:c r="F11" s="70" t="str">
+      <x:c r="F11" s="88" t="str">
         <x:v>Parallel-down compresses 12-month NII</x:v>
       </x:c>
       <x:c r="G11" s="1"/>
-      <x:c r="H11" s="142" t="str">
-        <x:v>3 | Review TRY duration hedge sizing: indicative pay-fixed IRS notional is TRY 10.3bn for a 50% DV01 reduction.</x:v>
-      </x:c>
-      <x:c r="I11" s="142"/>
-      <x:c r="J11" s="142"/>
-      <x:c r="K11" s="142"/>
-      <x:c r="L11" s="142"/>
+      <x:c r="H11" s="160" t="str">
+        <x:v>3 | Activate rapid-run readiness: the exploratory LCR proxy is 78.1%, stressed HQLA loses TRY 1.46bn and survival falls to 7 days.</x:v>
+      </x:c>
+      <x:c r="I11" s="160"/>
+      <x:c r="J11" s="160"/>
+      <x:c r="K11" s="160"/>
+      <x:c r="L11" s="160"/>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
       <x:c r="A12" s="1" t="str">
         <x:v>Combined LCR proxy</x:v>
       </x:c>
-      <x:c r="B12" s="69" t="n">
+      <x:c r="B12" s="87" t="n">
         <x:f>Liquidity!C4</x:f>
         <x:v>0.9483364199501884</x:v>
       </x:c>
-      <x:c r="C12" s="69" t="n">
+      <x:c r="C12" s="87" t="n">
         <x:f>Assumptions!B13</x:f>
         <x:v>1</x:v>
       </x:c>
@@ -2204,31 +2280,31 @@
         <x:f>IF(B12&gt;=C12,"WITHIN_LIMIT","BREACH")</x:f>
         <x:v>BREACH</x:v>
       </x:c>
-      <x:c r="F12" s="70" t="str">
+      <x:c r="F12" s="88" t="str">
         <x:v>Buffer falls below 100% in combined stress</x:v>
       </x:c>
       <x:c r="G12" s="1"/>
-      <x:c r="H12" s="142" t="str">
-        <x:v>4 | Protect NII downside: calibrate deposit beta and repricing lags before changing product pricing or hedge mix.</x:v>
-      </x:c>
-      <x:c r="I12" s="142"/>
-      <x:c r="J12" s="142"/>
-      <x:c r="K12" s="142"/>
-      <x:c r="L12" s="142"/>
+      <x:c r="H12" s="160" t="str">
+        <x:v>4 | Review TRY duration hedge sizing: indicative pay-fixed IRS notional is TRY 10.3bn for a 50% DV01 reduction.</x:v>
+      </x:c>
+      <x:c r="I12" s="160"/>
+      <x:c r="J12" s="160"/>
+      <x:c r="K12" s="160"/>
+      <x:c r="L12" s="160"/>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
       <x:c r="A13" s="1" t="str">
         <x:v>Combined survival days</x:v>
       </x:c>
-      <x:c r="B13" s="138" t="n">
+      <x:c r="B13" s="156" t="n">
         <x:f>Liquidity!G4</x:f>
         <x:v>30</x:v>
       </x:c>
-      <x:c r="C13" s="138" t="n">
+      <x:c r="C13" s="156" t="n">
         <x:f>Assumptions!B15</x:f>
         <x:v>30</x:v>
       </x:c>
-      <x:c r="D13" s="139" t="n">
+      <x:c r="D13" s="157" t="n">
         <x:f>B13-C13</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -2236,27 +2312,27 @@
         <x:f>IF(B13&gt;=C13,"WITHIN_LIMIT","BREACH")</x:f>
         <x:v>WITHIN_LIMIT</x:v>
       </x:c>
-      <x:c r="F13" s="70" t="str">
+      <x:c r="F13" s="88" t="str">
         <x:v>Exactly at management floor</x:v>
       </x:c>
       <x:c r="G13" s="1"/>
-      <x:c r="H13" s="142" t="str">
-        <x:v>5 | Treat every hedge output as a decision-support recommendation; treasury execution remains outside the model.</x:v>
-      </x:c>
-      <x:c r="I13" s="142"/>
-      <x:c r="J13" s="142"/>
-      <x:c r="K13" s="142"/>
-      <x:c r="L13" s="142"/>
+      <x:c r="H13" s="160" t="str">
+        <x:v>5 | Protect NII downside and treat every hedge output as decision support; execution remains outside the model.</x:v>
+      </x:c>
+      <x:c r="I13" s="160"/>
+      <x:c r="J13" s="160"/>
+      <x:c r="K13" s="160"/>
+      <x:c r="L13" s="160"/>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
       <x:c r="A14" s="1" t="str">
         <x:v>FX open / equity</x:v>
       </x:c>
-      <x:c r="B14" s="69" t="n">
+      <x:c r="B14" s="87" t="n">
         <x:f>'FX &amp; Hedge'!C4</x:f>
         <x:v>0.3333333333333333</x:v>
       </x:c>
-      <x:c r="C14" s="69" t="n">
+      <x:c r="C14" s="87" t="n">
         <x:f>Assumptions!B16</x:f>
         <x:v>0.2</x:v>
       </x:c>
@@ -2268,15 +2344,15 @@
         <x:f>IF(B14&lt;=C14,"WITHIN_LIMIT","BREACH")</x:f>
         <x:v>BREACH</x:v>
       </x:c>
-      <x:c r="F14" s="70" t="str">
+      <x:c r="F14" s="88" t="str">
         <x:v>USD short is the dominant remediable breach</x:v>
       </x:c>
       <x:c r="G14" s="1"/>
-      <x:c r="H14" s="142"/>
-      <x:c r="I14" s="142"/>
-      <x:c r="J14" s="142"/>
-      <x:c r="K14" s="142"/>
-      <x:c r="L14" s="142"/>
+      <x:c r="H14" s="160"/>
+      <x:c r="I14" s="160"/>
+      <x:c r="J14" s="160"/>
+      <x:c r="K14" s="160"/>
+      <x:c r="L14" s="160"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1"/>
@@ -2355,11 +2431,11 @@
         <x:f>'IRRBB EVE'!H6</x:f>
         <x:v>parallel_up</x:v>
       </x:c>
-      <x:c r="B19" s="143" t="n">
+      <x:c r="B19" s="161" t="n">
         <x:f>'IRRBB EVE'!I6</x:f>
         <x:v>-3092.3760850000035</x:v>
       </x:c>
-      <x:c r="C19" s="69" t="n">
+      <x:c r="C19" s="87" t="n">
         <x:f>'IRRBB EVE'!J6</x:f>
         <x:v>-0.13743893711111127</x:v>
       </x:c>
@@ -2371,12 +2447,12 @@
         <x:f>Liquidity!A8</x:f>
         <x:v>base</x:v>
       </x:c>
-      <x:c r="I19" s="69" t="n">
-        <x:f>Liquidity!F8</x:f>
+      <x:c r="I19" s="87" t="n">
+        <x:f>Liquidity!H8</x:f>
         <x:v>1.5872167592988458</x:v>
       </x:c>
       <x:c r="J19" s="33" t="n">
-        <x:f>Liquidity!G8</x:f>
+        <x:f>Liquidity!I8</x:f>
         <x:v>365</x:v>
       </x:c>
       <x:c r="K19" s="1"/>
@@ -2387,11 +2463,11 @@
         <x:f>'IRRBB EVE'!H7</x:f>
         <x:v>parallel_down</x:v>
       </x:c>
-      <x:c r="B20" s="143" t="n">
+      <x:c r="B20" s="161" t="n">
         <x:f>'IRRBB EVE'!I7</x:f>
         <x:v>3658.5116899999994</x:v>
       </x:c>
-      <x:c r="C20" s="69" t="n">
+      <x:c r="C20" s="87" t="n">
         <x:f>'IRRBB EVE'!J7</x:f>
         <x:v>0.16260051955555552</x:v>
       </x:c>
@@ -2403,12 +2479,12 @@
         <x:f>Liquidity!A9</x:f>
         <x:v>idiosyncratic</x:v>
       </x:c>
-      <x:c r="I20" s="69" t="n">
-        <x:f>Liquidity!F9</x:f>
+      <x:c r="I20" s="87" t="n">
+        <x:f>Liquidity!H9</x:f>
         <x:v>1.2021857923497268</x:v>
       </x:c>
       <x:c r="J20" s="33" t="n">
-        <x:f>Liquidity!G9</x:f>
+        <x:f>Liquidity!I9</x:f>
         <x:v>365</x:v>
       </x:c>
       <x:c r="K20" s="1"/>
@@ -2419,11 +2495,11 @@
         <x:f>'IRRBB EVE'!H8</x:f>
         <x:v>steepener</x:v>
       </x:c>
-      <x:c r="B21" s="143" t="n">
+      <x:c r="B21" s="161" t="n">
         <x:f>'IRRBB EVE'!I8</x:f>
         <x:v>-574.5688130000053</x:v>
       </x:c>
-      <x:c r="C21" s="69" t="n">
+      <x:c r="C21" s="87" t="n">
         <x:f>'IRRBB EVE'!J8</x:f>
         <x:v>-0.025536391688889125</x:v>
       </x:c>
@@ -2435,12 +2511,12 @@
         <x:f>Liquidity!A10</x:f>
         <x:v>market_wide</x:v>
       </x:c>
-      <x:c r="I21" s="69" t="n">
-        <x:f>Liquidity!F10</x:f>
+      <x:c r="I21" s="87" t="n">
+        <x:f>Liquidity!H10</x:f>
         <x:v>1.380496420935205</x:v>
       </x:c>
       <x:c r="J21" s="33" t="n">
-        <x:f>Liquidity!G10</x:f>
+        <x:f>Liquidity!I10</x:f>
         <x:v>365</x:v>
       </x:c>
       <x:c r="K21" s="1"/>
@@ -2451,11 +2527,11 @@
         <x:f>'IRRBB EVE'!H9</x:f>
         <x:v>flattener</x:v>
       </x:c>
-      <x:c r="B22" s="143" t="n">
+      <x:c r="B22" s="161" t="n">
         <x:f>'IRRBB EVE'!I9</x:f>
         <x:v>-96.98068100000091</x:v>
       </x:c>
-      <x:c r="C22" s="69" t="n">
+      <x:c r="C22" s="87" t="n">
         <x:f>'IRRBB EVE'!J9</x:f>
         <x:v>-0.00431025248888893</x:v>
       </x:c>
@@ -2467,12 +2543,12 @@
         <x:f>Liquidity!A11</x:f>
         <x:v>combined</x:v>
       </x:c>
-      <x:c r="I22" s="69" t="n">
-        <x:f>Liquidity!F11</x:f>
+      <x:c r="I22" s="87" t="n">
+        <x:f>Liquidity!H11</x:f>
         <x:v>0.9483364199501884</x:v>
       </x:c>
       <x:c r="J22" s="33" t="n">
-        <x:f>Liquidity!G11</x:f>
+        <x:f>Liquidity!I11</x:f>
         <x:v>30</x:v>
       </x:c>
       <x:c r="K22" s="1"/>
@@ -2483,11 +2559,11 @@
         <x:f>'IRRBB EVE'!H10</x:f>
         <x:v>short_up</x:v>
       </x:c>
-      <x:c r="B23" s="143" t="n">
+      <x:c r="B23" s="161" t="n">
         <x:f>'IRRBB EVE'!I10</x:f>
         <x:v>-1362.5024140000023</x:v>
       </x:c>
-      <x:c r="C23" s="69" t="n">
+      <x:c r="C23" s="87" t="n">
         <x:f>'IRRBB EVE'!J10</x:f>
         <x:v>-0.060555662844444545</x:v>
       </x:c>
@@ -2495,9 +2571,18 @@
       <x:c r="E23" s="1"/>
       <x:c r="F23" s="1"/>
       <x:c r="G23" s="1"/>
-      <x:c r="H23" s="1"/>
-      <x:c r="I23" s="1"/>
-      <x:c r="J23" s="1"/>
+      <x:c r="H23" s="33" t="str">
+        <x:f>Liquidity!A12</x:f>
+        <x:v>rapid_digital_run</x:v>
+      </x:c>
+      <x:c r="I23" s="87" t="n">
+        <x:f>Liquidity!H12</x:f>
+        <x:v>0.7809151560078172</x:v>
+      </x:c>
+      <x:c r="J23" s="33" t="n">
+        <x:f>Liquidity!I12</x:f>
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="K23" s="1"/>
       <x:c r="L23" s="1"/>
     </x:row>
@@ -2506,11 +2591,11 @@
         <x:f>'IRRBB EVE'!H11</x:f>
         <x:v>short_down</x:v>
       </x:c>
-      <x:c r="B24" s="143" t="n">
+      <x:c r="B24" s="161" t="n">
         <x:f>'IRRBB EVE'!I11</x:f>
         <x:v>1462.7598829999988</x:v>
       </x:c>
-      <x:c r="C24" s="69" t="n">
+      <x:c r="C24" s="87" t="n">
         <x:f>'IRRBB EVE'!J11</x:f>
         <x:v>0.0650115503555555</x:v>
       </x:c>
@@ -3343,7 +3428,7 @@
     <x:cfRule type="containsText" dxfId="24" priority="5" operator="containsText" text="OK"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30022f37619347c8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R282e6f778e974f2d"/>
 </x:worksheet>
 </file>
 
@@ -4115,11 +4200,11 @@
         <x:v>Official/method sources</x:v>
       </x:c>
       <x:c r="B27" s="33" t="n">
-        <x:f>COUNTA(Sources!A5:A12)</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTA(Sources!A5:A13)</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C27" s="1" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D27" s="1" t="n">
         <x:f>B27-C27</x:f>
@@ -4190,18 +4275,18 @@
       <x:c r="M29" s="1"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="74" t="str">
+      <x:c r="A30" s="92" t="str">
         <x:v>MODEL STATUS</x:v>
       </x:c>
-      <x:c r="B30" s="75"/>
-      <x:c r="C30" s="75"/>
-      <x:c r="D30" s="75"/>
-      <x:c r="E30" s="75"/>
-      <x:c r="F30" s="75" t="str">
+      <x:c r="B30" s="93"/>
+      <x:c r="C30" s="93"/>
+      <x:c r="D30" s="93"/>
+      <x:c r="E30" s="93"/>
+      <x:c r="F30" s="93" t="str">
         <x:f>IF(COUNTIF(F21:F28,"FAIL")=0,"OK - RISK FLAGS SURFACED","REVIEW REQUIRED")</x:f>
         <x:v>OK - RISK FLAGS SURFACED</x:v>
       </x:c>
-      <x:c r="G30" s="76"/>
+      <x:c r="G30" s="94"/>
       <x:c r="H30" s="1"/>
       <x:c r="I30" s="1"/>
       <x:c r="J30" s="1"/>
@@ -5092,7 +5177,7 @@
       <x:c r="C5" s="1" t="str">
         <x:v>2026-01-01</x:v>
       </x:c>
-      <x:c r="D5" s="70" t="str">
+      <x:c r="D5" s="88" t="str">
         <x:v>TRY 400/500/300; USD 200/300/225; EUR 225/350/200</x:v>
       </x:c>
       <x:c r="E5" s="1" t="str">
@@ -5101,13 +5186,13 @@
       <x:c r="F5" s="1" t="str">
         <x:v>Basel Committee on Banking Supervision</x:v>
       </x:c>
-      <x:c r="G5" s="70" t="str">
+      <x:c r="G5" s="88" t="str">
         <x:v>https://www.bis.org/bcbs/publ/d578.pdf</x:v>
       </x:c>
-      <x:c r="H5" s="70" t="str">
+      <x:c r="H5" s="88" t="str">
         <x:v>official_methodology</x:v>
       </x:c>
-      <x:c r="I5" s="70" t="str">
+      <x:c r="I5" s="88" t="str">
         <x:v>Revised shocks implemented from 1 January 2026</x:v>
       </x:c>
     </x:row>
@@ -5121,7 +5206,7 @@
       <x:c r="C6" s="1" t="str">
         <x:v>current framework</x:v>
       </x:c>
-      <x:c r="D6" s="70" t="str">
+      <x:c r="D6" s="88" t="str">
         <x:v>HQLA / 30-day net cash outflows</x:v>
       </x:c>
       <x:c r="E6" s="1" t="str">
@@ -5130,13 +5215,13 @@
       <x:c r="F6" s="1" t="str">
         <x:v>Bank for International Settlements</x:v>
       </x:c>
-      <x:c r="G6" s="70" t="str">
+      <x:c r="G6" s="88" t="str">
         <x:v>https://www.bis.org/basel_framework/chapter/LCR/20.htm</x:v>
       </x:c>
-      <x:c r="H6" s="70" t="str">
+      <x:c r="H6" s="88" t="str">
         <x:v>official_methodology</x:v>
       </x:c>
-      <x:c r="I6" s="70" t="str">
+      <x:c r="I6" s="88" t="str">
         <x:v>Workbook output is labelled proxy, not a regulatory return</x:v>
       </x:c>
     </x:row>
@@ -5150,7 +5235,7 @@
       <x:c r="C7" s="1" t="str">
         <x:v>current framework</x:v>
       </x:c>
-      <x:c r="D7" s="70" t="str">
+      <x:c r="D7" s="88" t="str">
         <x:v>ASF / RSF</x:v>
       </x:c>
       <x:c r="E7" s="1" t="str">
@@ -5159,13 +5244,13 @@
       <x:c r="F7" s="1" t="str">
         <x:v>Bank for International Settlements</x:v>
       </x:c>
-      <x:c r="G7" s="70" t="str">
+      <x:c r="G7" s="88" t="str">
         <x:v>https://www.bis.org/basel_framework/chapter/NSF/20.htm</x:v>
       </x:c>
-      <x:c r="H7" s="70" t="str">
+      <x:c r="H7" s="88" t="str">
         <x:v>official_methodology</x:v>
       </x:c>
-      <x:c r="I7" s="70" t="str">
+      <x:c r="I7" s="88" t="str">
         <x:v>Workbook output is labelled proxy, not a regulatory return</x:v>
       </x:c>
     </x:row>
@@ -5179,7 +5264,7 @@
       <x:c r="C8" s="1" t="str">
         <x:v>2026-08-19</x:v>
       </x:c>
-      <x:c r="D8" s="70" t="n">
+      <x:c r="D8" s="88" t="n">
         <x:v>0.37</x:v>
       </x:c>
       <x:c r="E8" s="1" t="str">
@@ -5188,13 +5273,13 @@
       <x:c r="F8" s="1" t="str">
         <x:v>TCMB</x:v>
       </x:c>
-      <x:c r="G8" s="70" t="str">
+      <x:c r="G8" s="88" t="str">
         <x:v>https://www.tcmb.gov.tr/wps/wcm/connect/tr/tcmb+tr/main+menu/duyurular/basin/2026/duy2026-23</x:v>
       </x:c>
-      <x:c r="H8" s="70" t="str">
+      <x:c r="H8" s="88" t="str">
         <x:v>official_observation</x:v>
       </x:c>
-      <x:c r="I8" s="70" t="str">
+      <x:c r="I8" s="88" t="str">
         <x:v>Reference market context; not used as a bank position</x:v>
       </x:c>
     </x:row>
@@ -5208,7 +5293,7 @@
       <x:c r="C9" s="1" t="str">
         <x:v>2026-08-19</x:v>
       </x:c>
-      <x:c r="D9" s="70" t="n">
+      <x:c r="D9" s="88" t="n">
         <x:v>47.8467</x:v>
       </x:c>
       <x:c r="E9" s="1" t="str">
@@ -5217,13 +5302,13 @@
       <x:c r="F9" s="1" t="str">
         <x:v>TCMB via e-Devlet</x:v>
       </x:c>
-      <x:c r="G9" s="70" t="str">
+      <x:c r="G9" s="88" t="str">
         <x:v>https://www.turkiye.gov.tr/doviz-kurlari</x:v>
       </x:c>
-      <x:c r="H9" s="70" t="str">
+      <x:c r="H9" s="88" t="str">
         <x:v>official_observation</x:v>
       </x:c>
-      <x:c r="I9" s="70" t="str">
+      <x:c r="I9" s="88" t="str">
         <x:v>Public market observation</x:v>
       </x:c>
     </x:row>
@@ -5237,7 +5322,7 @@
       <x:c r="C10" s="1" t="str">
         <x:v>2026-08-19</x:v>
       </x:c>
-      <x:c r="D10" s="70" t="n">
+      <x:c r="D10" s="88" t="n">
         <x:v>55.5061</x:v>
       </x:c>
       <x:c r="E10" s="1" t="str">
@@ -5246,13 +5331,13 @@
       <x:c r="F10" s="1" t="str">
         <x:v>TCMB via e-Devlet</x:v>
       </x:c>
-      <x:c r="G10" s="70" t="str">
+      <x:c r="G10" s="88" t="str">
         <x:v>https://www.turkiye.gov.tr/doviz-kurlari</x:v>
       </x:c>
-      <x:c r="H10" s="70" t="str">
+      <x:c r="H10" s="88" t="str">
         <x:v>official_observation</x:v>
       </x:c>
-      <x:c r="I10" s="70" t="str">
+      <x:c r="I10" s="88" t="str">
         <x:v>Public market observation</x:v>
       </x:c>
     </x:row>
@@ -5266,7 +5351,7 @@
       <x:c r="C11" s="1" t="str">
         <x:v>2026-06-30</x:v>
       </x:c>
-      <x:c r="D11" s="70" t="str">
+      <x:c r="D11" s="88" t="str">
         <x:v>Assets 52,727,562; loans 26,791,320; deposits 30,109,453</x:v>
       </x:c>
       <x:c r="E11" s="1" t="str">
@@ -5275,13 +5360,13 @@
       <x:c r="F11" s="1" t="str">
         <x:v>BDDK</x:v>
       </x:c>
-      <x:c r="G11" s="70" t="str">
+      <x:c r="G11" s="88" t="str">
         <x:v>https://www.bddk.org.tr/BultenAylik/tr/Home/HaberBulteni</x:v>
       </x:c>
-      <x:c r="H11" s="70" t="str">
+      <x:c r="H11" s="88" t="str">
         <x:v>official_benchmark</x:v>
       </x:c>
-      <x:c r="I11" s="70" t="str">
+      <x:c r="I11" s="88" t="str">
         <x:v>Contextual benchmark only; Aurelia bank is fictional</x:v>
       </x:c>
     </x:row>
@@ -5295,7 +5380,7 @@
       <x:c r="C12" s="1" t="str">
         <x:v>2026-08-19</x:v>
       </x:c>
-      <x:c r="D12" s="70" t="str">
+      <x:c r="D12" s="88" t="str">
         <x:v>Deterministic seed 20260819</x:v>
       </x:c>
       <x:c r="E12" s="1" t="str">
@@ -5304,26 +5389,44 @@
       <x:c r="F12" s="1" t="str">
         <x:v>Project generator</x:v>
       </x:c>
-      <x:c r="G12" s="70" t="str">
+      <x:c r="G12" s="88" t="str">
         <x:v>docs/data_provenance.md</x:v>
       </x:c>
-      <x:c r="H12" s="70" t="str">
+      <x:c r="H12" s="88" t="str">
         <x:v>controlled_synthetic</x:v>
       </x:c>
-      <x:c r="I12" s="70" t="str">
+      <x:c r="I12" s="88" t="str">
         <x:v>No customer data, PII or confidential bank data</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="1"/>
-      <x:c r="B13" s="1"/>
-      <x:c r="C13" s="1"/>
-      <x:c r="D13" s="1"/>
-      <x:c r="E13" s="1"/>
-      <x:c r="F13" s="1"/>
-      <x:c r="G13" s="1"/>
-      <x:c r="H13" s="1"/>
-      <x:c r="I13" s="1"/>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="1" t="str">
+        <x:v>AURELIA-DIGITAL-RUN</x:v>
+      </x:c>
+      <x:c r="B13" s="1" t="str">
+        <x:v>Rapid digital deposit-run assumptions</x:v>
+      </x:c>
+      <x:c r="C13" s="1" t="str">
+        <x:v>2026-08-21</x:v>
+      </x:c>
+      <x:c r="D13" s="88" t="str">
+        <x:v>45% demand; 30% term; 55% day 1; 85% day 7</x:v>
+      </x:c>
+      <x:c r="E13" s="1" t="str">
+        <x:v>scenario parameters</x:v>
+      </x:c>
+      <x:c r="F13" s="1" t="str">
+        <x:v>Internal ALCO demonstration scenario</x:v>
+      </x:c>
+      <x:c r="G13" s="88" t="str">
+        <x:v>docs/rapid_digital_run_scenario.md</x:v>
+      </x:c>
+      <x:c r="H13" s="88" t="str">
+        <x:v>controlled_internal_assumption</x:v>
+      </x:c>
+      <x:c r="I13" s="88" t="str">
+        <x:v>Severe exploratory vulnerability test; not a forecast or regulatory calibration</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1"/>
@@ -7187,7 +7290,7 @@
     <x:mergeCell ref="E12:J12"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31f625cb559148df"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4522e2ee601d49ec"/>
 </x:worksheet>
 </file>
 
@@ -19046,7 +19149,7 @@
     <x:mergeCell ref="A4:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re583719015c5427a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40f6aec535884b7d"/>
 </x:worksheet>
 </file>
 
@@ -19911,7 +20014,7 @@
     <x:mergeCell ref="A4:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6664cecc1c2d41de"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55524bdc76794467"/>
 </x:worksheet>
 </file>
 
@@ -19919,16 +20022,18 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -19944,10 +20049,15 @@
       <x:c r="H1" s="4"/>
       <x:c r="I1" s="4"/>
       <x:c r="J1" s="4"/>
+      <x:c r="K1" s="4"/>
+      <x:c r="L1" s="4"/>
+      <x:c r="M1" s="1"/>
+      <x:c r="N1" s="1"/>
+      <x:c r="O1" s="1"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>LCR and NSFR proxy analytics for portfolio demonstration; not a regulatory return</x:v>
+        <x:v>Five governed management scenarios including a severe rapid digital run; not a regulatory return</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -19958,6 +20068,11 @@
       <x:c r="H2" s="7"/>
       <x:c r="I2" s="7"/>
       <x:c r="J2" s="7"/>
+      <x:c r="K2" s="7"/>
+      <x:c r="L2" s="7"/>
+      <x:c r="M2" s="1"/>
+      <x:c r="N2" s="1"/>
+      <x:c r="O2" s="1"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1"/>
@@ -19970,6 +20085,11 @@
       <x:c r="H3" s="1"/>
       <x:c r="I3" s="1"/>
       <x:c r="J3" s="1"/>
+      <x:c r="K3" s="1"/>
+      <x:c r="L3" s="1"/>
+      <x:c r="M3" s="1"/>
+      <x:c r="N3" s="1"/>
+      <x:c r="O3" s="1"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="61" t="str">
@@ -19977,7 +20097,7 @@
       </x:c>
       <x:c r="B4" s="62"/>
       <x:c r="C4" s="63" t="n">
-        <x:f>F11</x:f>
+        <x:f>H11</x:f>
         <x:v>0.9483364199501884</x:v>
       </x:c>
       <x:c r="D4" s="1"/>
@@ -19986,12 +20106,22 @@
       </x:c>
       <x:c r="F4" s="67"/>
       <x:c r="G4" s="68" t="n">
-        <x:f>G11</x:f>
+        <x:f>I11</x:f>
         <x:v>30</x:v>
       </x:c>
       <x:c r="H4" s="1"/>
-      <x:c r="I4" s="1"/>
-      <x:c r="J4" s="1"/>
+      <x:c r="I4" s="79" t="str">
+        <x:v>Rapid-run LCR proxy</x:v>
+      </x:c>
+      <x:c r="J4" s="80"/>
+      <x:c r="K4" s="81" t="n">
+        <x:f>H12</x:f>
+        <x:v>0.7809151560078172</x:v>
+      </x:c>
+      <x:c r="L4" s="82"/>
+      <x:c r="M4" s="1"/>
+      <x:c r="N4" s="1"/>
+      <x:c r="O4" s="1"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="1"/>
@@ -20002,8 +20132,18 @@
       <x:c r="F5" s="1"/>
       <x:c r="G5" s="1"/>
       <x:c r="H5" s="1"/>
-      <x:c r="I5" s="1"/>
-      <x:c r="J5" s="1"/>
+      <x:c r="I5" s="83" t="str">
+        <x:v>Rapid-run survival</x:v>
+      </x:c>
+      <x:c r="J5" s="84"/>
+      <x:c r="K5" s="85" t="n">
+        <x:f>I12</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="L5" s="86"/>
+      <x:c r="M5" s="1"/>
+      <x:c r="N5" s="1"/>
+      <x:c r="O5" s="1"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="1"/>
@@ -20016,42 +20156,54 @@
       <x:c r="H6" s="1"/>
       <x:c r="I6" s="1"/>
       <x:c r="J6" s="1"/>
+      <x:c r="K6" s="1"/>
+      <x:c r="L6" s="1"/>
+      <x:c r="M6" s="1"/>
+      <x:c r="N6" s="1"/>
+      <x:c r="O6" s="1"/>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="24" t="str">
         <x:v>Scenario</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>HQLA</x:v>
+        <x:v>Base HQLA</x:v>
       </x:c>
       <x:c r="C7" s="24" t="str">
+        <x:v>Stressed HQLA</x:v>
+      </x:c>
+      <x:c r="D7" s="24" t="str">
+        <x:v>HQLA MV loss</x:v>
+      </x:c>
+      <x:c r="E7" s="24" t="str">
         <x:v>Gross outflows 30d</x:v>
       </x:c>
-      <x:c r="D7" s="24" t="str">
+      <x:c r="F7" s="24" t="str">
         <x:v>Eligible inflows 30d</x:v>
       </x:c>
-      <x:c r="E7" s="24" t="str">
+      <x:c r="G7" s="24" t="str">
         <x:v>Net outflows 30d</x:v>
       </x:c>
-      <x:c r="F7" s="24" t="str">
+      <x:c r="H7" s="24" t="str">
         <x:v>LCR proxy</x:v>
       </x:c>
-      <x:c r="G7" s="24" t="str">
+      <x:c r="I7" s="24" t="str">
         <x:v>Survival days</x:v>
       </x:c>
-      <x:c r="H7" s="24" t="str">
+      <x:c r="J7" s="24" t="str">
         <x:v>ASF</x:v>
       </x:c>
-      <x:c r="I7" s="24" t="str">
+      <x:c r="K7" s="24" t="str">
         <x:v>RSF</x:v>
       </x:c>
-      <x:c r="J7" s="24" t="str">
+      <x:c r="L7" s="24" t="str">
         <x:v>NSFR proxy</x:v>
       </x:c>
-      <x:c r="L7" t="str">
+      <x:c r="M7" s="1"/>
+      <x:c r="N7" s="1" t="str">
         <x:v>Scenario</x:v>
       </x:c>
-      <x:c r="M7" t="str">
+      <x:c r="O7" s="1" t="str">
         <x:v>LCR proxy</x:v>
       </x:c>
     </x:row>
@@ -20063,38 +20215,46 @@
         <x:v>59400</x:v>
       </x:c>
       <x:c r="C8" s="13" t="n">
+        <x:v>59400</x:v>
+      </x:c>
+      <x:c r="D8" s="13" t="n">
+        <x:f>B8-C8</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="13" t="n">
         <x:v>37424</x:v>
       </x:c>
-      <x:c r="D8" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E8" s="13" t="n">
-        <x:f>C8-MIN(D8,C8*75%)</x:f>
+      <x:c r="F8" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="13" t="n">
+        <x:f>E8-MIN(F8,E8*75%)</x:f>
         <x:v>37424</x:v>
       </x:c>
-      <x:c r="F8" s="11" t="n">
-        <x:f>B8/E8</x:f>
+      <x:c r="H8" s="11" t="n">
+        <x:f>C8/G8</x:f>
         <x:v>1.5872167592988458</x:v>
       </x:c>
-      <x:c r="G8" s="1" t="n">
+      <x:c r="I8" s="1" t="n">
         <x:v>365</x:v>
       </x:c>
-      <x:c r="H8" s="13" t="n">
+      <x:c r="J8" s="13" t="n">
         <x:v>150450</x:v>
       </x:c>
-      <x:c r="I8" s="13" t="n">
+      <x:c r="K8" s="13" t="n">
         <x:v>104950</x:v>
       </x:c>
-      <x:c r="J8" s="11" t="n">
-        <x:f>H8/I8</x:f>
+      <x:c r="L8" s="11" t="n">
+        <x:f>J8/K8</x:f>
         <x:v>1.4335397808480228</x:v>
       </x:c>
-      <x:c r="L8" t="str">
+      <x:c r="M8" s="1"/>
+      <x:c r="N8" s="1" t="str">
         <x:f>A8</x:f>
         <x:v>base</x:v>
       </x:c>
-      <x:c r="M8" t="n">
-        <x:f>F8</x:f>
+      <x:c r="O8" s="1" t="n">
+        <x:f>H8</x:f>
         <x:v>1.5872167592988458</x:v>
       </x:c>
     </x:row>
@@ -20106,38 +20266,46 @@
         <x:v>59400</x:v>
       </x:c>
       <x:c r="C9" s="13" t="n">
+        <x:v>59400</x:v>
+      </x:c>
+      <x:c r="D9" s="13" t="n">
+        <x:f>B9-C9</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="13" t="n">
         <x:v>49410</x:v>
       </x:c>
-      <x:c r="D9" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E9" s="13" t="n">
-        <x:f>C9-MIN(D9,C9*75%)</x:f>
+      <x:c r="F9" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="13" t="n">
+        <x:f>E9-MIN(F9,E9*75%)</x:f>
         <x:v>49410</x:v>
       </x:c>
-      <x:c r="F9" s="11" t="n">
-        <x:f>B9/E9</x:f>
+      <x:c r="H9" s="11" t="n">
+        <x:f>C9/G9</x:f>
         <x:v>1.2021857923497268</x:v>
       </x:c>
-      <x:c r="G9" s="1" t="n">
+      <x:c r="I9" s="1" t="n">
         <x:v>365</x:v>
       </x:c>
-      <x:c r="H9" s="13" t="n">
+      <x:c r="J9" s="13" t="n">
         <x:v>150450</x:v>
       </x:c>
-      <x:c r="I9" s="13" t="n">
+      <x:c r="K9" s="13" t="n">
         <x:v>104950</x:v>
       </x:c>
-      <x:c r="J9" s="11" t="n">
-        <x:f>H9/I9</x:f>
+      <x:c r="L9" s="11" t="n">
+        <x:f>J9/K9</x:f>
         <x:v>1.4335397808480228</x:v>
       </x:c>
-      <x:c r="L9" t="str">
+      <x:c r="M9" s="1"/>
+      <x:c r="N9" s="1" t="str">
         <x:f>A9</x:f>
         <x:v>idiosyncratic</x:v>
       </x:c>
-      <x:c r="M9" t="n">
-        <x:f>F9</x:f>
+      <x:c r="O9" s="1" t="n">
+        <x:f>H9</x:f>
         <x:v>1.2021857923497268</x:v>
       </x:c>
     </x:row>
@@ -20149,38 +20317,46 @@
         <x:v>59400</x:v>
       </x:c>
       <x:c r="C10" s="13" t="n">
+        <x:v>59400</x:v>
+      </x:c>
+      <x:c r="D10" s="13" t="n">
+        <x:f>B10-C10</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="13" t="n">
         <x:v>43028</x:v>
       </x:c>
-      <x:c r="D10" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E10" s="13" t="n">
-        <x:f>C10-MIN(D10,C10*75%)</x:f>
+      <x:c r="F10" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" s="13" t="n">
+        <x:f>E10-MIN(F10,E10*75%)</x:f>
         <x:v>43028</x:v>
       </x:c>
-      <x:c r="F10" s="11" t="n">
-        <x:f>B10/E10</x:f>
+      <x:c r="H10" s="11" t="n">
+        <x:f>C10/G10</x:f>
         <x:v>1.380496420935205</x:v>
       </x:c>
-      <x:c r="G10" s="1" t="n">
+      <x:c r="I10" s="1" t="n">
         <x:v>365</x:v>
       </x:c>
-      <x:c r="H10" s="13" t="n">
+      <x:c r="J10" s="13" t="n">
         <x:v>150450</x:v>
       </x:c>
-      <x:c r="I10" s="13" t="n">
+      <x:c r="K10" s="13" t="n">
         <x:v>104950</x:v>
       </x:c>
-      <x:c r="J10" s="11" t="n">
-        <x:f>H10/I10</x:f>
+      <x:c r="L10" s="11" t="n">
+        <x:f>J10/K10</x:f>
         <x:v>1.4335397808480228</x:v>
       </x:c>
-      <x:c r="L10" t="str">
+      <x:c r="M10" s="1"/>
+      <x:c r="N10" s="1" t="str">
         <x:f>A10</x:f>
         <x:v>market_wide</x:v>
       </x:c>
-      <x:c r="M10" t="n">
-        <x:f>F10</x:f>
+      <x:c r="O10" s="1" t="n">
+        <x:f>H10</x:f>
         <x:v>1.380496420935205</x:v>
       </x:c>
     </x:row>
@@ -20192,52 +20368,99 @@
         <x:v>59400</x:v>
       </x:c>
       <x:c r="C11" s="13" t="n">
+        <x:v>59400</x:v>
+      </x:c>
+      <x:c r="D11" s="13" t="n">
+        <x:f>B11-C11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="13" t="n">
         <x:v>62636</x:v>
       </x:c>
-      <x:c r="D11" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E11" s="13" t="n">
-        <x:f>C11-MIN(D11,C11*75%)</x:f>
+      <x:c r="F11" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G11" s="13" t="n">
+        <x:f>E11-MIN(F11,E11*75%)</x:f>
         <x:v>62636</x:v>
       </x:c>
-      <x:c r="F11" s="11" t="n">
-        <x:f>B11/E11</x:f>
+      <x:c r="H11" s="11" t="n">
+        <x:f>C11/G11</x:f>
         <x:v>0.9483364199501884</x:v>
       </x:c>
-      <x:c r="G11" s="1" t="n">
+      <x:c r="I11" s="1" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="H11" s="13" t="n">
+      <x:c r="J11" s="13" t="n">
         <x:v>150450</x:v>
       </x:c>
-      <x:c r="I11" s="13" t="n">
+      <x:c r="K11" s="13" t="n">
         <x:v>104950</x:v>
       </x:c>
-      <x:c r="J11" s="11" t="n">
-        <x:f>H11/I11</x:f>
+      <x:c r="L11" s="11" t="n">
+        <x:f>J11/K11</x:f>
         <x:v>1.4335397808480228</x:v>
       </x:c>
-      <x:c r="L11" t="str">
+      <x:c r="M11" s="1"/>
+      <x:c r="N11" s="1" t="str">
         <x:f>A11</x:f>
         <x:v>combined</x:v>
       </x:c>
-      <x:c r="M11" t="n">
-        <x:f>F11</x:f>
+      <x:c r="O11" s="1" t="n">
+        <x:f>H11</x:f>
         <x:v>0.9483364199501884</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="1"/>
-      <x:c r="B12" s="1"/>
-      <x:c r="C12" s="1"/>
-      <x:c r="D12" s="1"/>
-      <x:c r="E12" s="1"/>
-      <x:c r="F12" s="1"/>
-      <x:c r="G12" s="1"/>
-      <x:c r="H12" s="1"/>
-      <x:c r="I12" s="1"/>
-      <x:c r="J12" s="1"/>
+      <x:c r="A12" s="1" t="str">
+        <x:v>rapid_digital_run</x:v>
+      </x:c>
+      <x:c r="B12" s="13" t="n">
+        <x:v>59400</x:v>
+      </x:c>
+      <x:c r="C12" s="13" t="n">
+        <x:v>57940</x:v>
+      </x:c>
+      <x:c r="D12" s="13" t="n">
+        <x:f>B12-C12</x:f>
+        <x:v>1460</x:v>
+      </x:c>
+      <x:c r="E12" s="13" t="n">
+        <x:v>74195</x:v>
+      </x:c>
+      <x:c r="F12" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" s="13" t="n">
+        <x:f>E12-MIN(F12,E12*75%)</x:f>
+        <x:v>74195</x:v>
+      </x:c>
+      <x:c r="H12" s="11" t="n">
+        <x:f>C12/G12</x:f>
+        <x:v>0.7809151560078172</x:v>
+      </x:c>
+      <x:c r="I12" s="1" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J12" s="13" t="n">
+        <x:v>150450</x:v>
+      </x:c>
+      <x:c r="K12" s="13" t="n">
+        <x:v>104950</x:v>
+      </x:c>
+      <x:c r="L12" s="11" t="n">
+        <x:f>J12/K12</x:f>
+        <x:v>1.4335397808480228</x:v>
+      </x:c>
+      <x:c r="M12" s="1"/>
+      <x:c r="N12" s="1" t="str">
+        <x:f>A12</x:f>
+        <x:v>rapid_digital_run</x:v>
+      </x:c>
+      <x:c r="O12" s="1" t="n">
+        <x:f>H12</x:f>
+        <x:v>0.7809151560078172</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1"/>
@@ -20250,6 +20473,11 @@
       <x:c r="H13" s="1"/>
       <x:c r="I13" s="1"/>
       <x:c r="J13" s="1"/>
+      <x:c r="K13" s="1"/>
+      <x:c r="L13" s="1"/>
+      <x:c r="M13" s="1"/>
+      <x:c r="N13" s="1"/>
+      <x:c r="O13" s="1"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1"/>
@@ -20262,6 +20490,11 @@
       <x:c r="H14" s="1"/>
       <x:c r="I14" s="1"/>
       <x:c r="J14" s="1"/>
+      <x:c r="K14" s="1"/>
+      <x:c r="L14" s="1"/>
+      <x:c r="M14" s="1"/>
+      <x:c r="N14" s="1"/>
+      <x:c r="O14" s="1"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1"/>
@@ -20274,6 +20507,11 @@
       <x:c r="H15" s="1"/>
       <x:c r="I15" s="1"/>
       <x:c r="J15" s="1"/>
+      <x:c r="K15" s="1"/>
+      <x:c r="L15" s="1"/>
+      <x:c r="M15" s="1"/>
+      <x:c r="N15" s="1"/>
+      <x:c r="O15" s="1"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1"/>
@@ -20286,6 +20524,11 @@
       <x:c r="H16" s="1"/>
       <x:c r="I16" s="1"/>
       <x:c r="J16" s="1"/>
+      <x:c r="K16" s="1"/>
+      <x:c r="L16" s="1"/>
+      <x:c r="M16" s="1"/>
+      <x:c r="N16" s="1"/>
+      <x:c r="O16" s="1"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="1"/>
@@ -20298,6 +20541,11 @@
       <x:c r="H17" s="1"/>
       <x:c r="I17" s="1"/>
       <x:c r="J17" s="1"/>
+      <x:c r="K17" s="1"/>
+      <x:c r="L17" s="1"/>
+      <x:c r="M17" s="1"/>
+      <x:c r="N17" s="1"/>
+      <x:c r="O17" s="1"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="1"/>
@@ -20310,6 +20558,11 @@
       <x:c r="H18" s="1"/>
       <x:c r="I18" s="1"/>
       <x:c r="J18" s="1"/>
+      <x:c r="K18" s="1"/>
+      <x:c r="L18" s="1"/>
+      <x:c r="M18" s="1"/>
+      <x:c r="N18" s="1"/>
+      <x:c r="O18" s="1"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="1"/>
@@ -20322,6 +20575,11 @@
       <x:c r="H19" s="1"/>
       <x:c r="I19" s="1"/>
       <x:c r="J19" s="1"/>
+      <x:c r="K19" s="1"/>
+      <x:c r="L19" s="1"/>
+      <x:c r="M19" s="1"/>
+      <x:c r="N19" s="1"/>
+      <x:c r="O19" s="1"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="1"/>
@@ -20334,6 +20592,11 @@
       <x:c r="H20" s="1"/>
       <x:c r="I20" s="1"/>
       <x:c r="J20" s="1"/>
+      <x:c r="K20" s="1"/>
+      <x:c r="L20" s="1"/>
+      <x:c r="M20" s="1"/>
+      <x:c r="N20" s="1"/>
+      <x:c r="O20" s="1"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="1"/>
@@ -20346,6 +20609,11 @@
       <x:c r="H21" s="1"/>
       <x:c r="I21" s="1"/>
       <x:c r="J21" s="1"/>
+      <x:c r="K21" s="1"/>
+      <x:c r="L21" s="1"/>
+      <x:c r="M21" s="1"/>
+      <x:c r="N21" s="1"/>
+      <x:c r="O21" s="1"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="1"/>
@@ -20358,6 +20626,11 @@
       <x:c r="H22" s="1"/>
       <x:c r="I22" s="1"/>
       <x:c r="J22" s="1"/>
+      <x:c r="K22" s="1"/>
+      <x:c r="L22" s="1"/>
+      <x:c r="M22" s="1"/>
+      <x:c r="N22" s="1"/>
+      <x:c r="O22" s="1"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="1"/>
@@ -20370,6 +20643,11 @@
       <x:c r="H23" s="1"/>
       <x:c r="I23" s="1"/>
       <x:c r="J23" s="1"/>
+      <x:c r="K23" s="1"/>
+      <x:c r="L23" s="1"/>
+      <x:c r="M23" s="1"/>
+      <x:c r="N23" s="1"/>
+      <x:c r="O23" s="1"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="1"/>
@@ -20382,6 +20660,11 @@
       <x:c r="H24" s="1"/>
       <x:c r="I24" s="1"/>
       <x:c r="J24" s="1"/>
+      <x:c r="K24" s="1"/>
+      <x:c r="L24" s="1"/>
+      <x:c r="M24" s="1"/>
+      <x:c r="N24" s="1"/>
+      <x:c r="O24" s="1"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="1"/>
@@ -20394,6 +20677,11 @@
       <x:c r="H25" s="1"/>
       <x:c r="I25" s="1"/>
       <x:c r="J25" s="1"/>
+      <x:c r="K25" s="1"/>
+      <x:c r="L25" s="1"/>
+      <x:c r="M25" s="1"/>
+      <x:c r="N25" s="1"/>
+      <x:c r="O25" s="1"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="1"/>
@@ -20406,6 +20694,11 @@
       <x:c r="H26" s="1"/>
       <x:c r="I26" s="1"/>
       <x:c r="J26" s="1"/>
+      <x:c r="K26" s="1"/>
+      <x:c r="L26" s="1"/>
+      <x:c r="M26" s="1"/>
+      <x:c r="N26" s="1"/>
+      <x:c r="O26" s="1"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="1"/>
@@ -20418,6 +20711,11 @@
       <x:c r="H27" s="1"/>
       <x:c r="I27" s="1"/>
       <x:c r="J27" s="1"/>
+      <x:c r="K27" s="1"/>
+      <x:c r="L27" s="1"/>
+      <x:c r="M27" s="1"/>
+      <x:c r="N27" s="1"/>
+      <x:c r="O27" s="1"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="1"/>
@@ -20430,6 +20728,11 @@
       <x:c r="H28" s="1"/>
       <x:c r="I28" s="1"/>
       <x:c r="J28" s="1"/>
+      <x:c r="K28" s="1"/>
+      <x:c r="L28" s="1"/>
+      <x:c r="M28" s="1"/>
+      <x:c r="N28" s="1"/>
+      <x:c r="O28" s="1"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="1"/>
@@ -20442,6 +20745,11 @@
       <x:c r="H29" s="1"/>
       <x:c r="I29" s="1"/>
       <x:c r="J29" s="1"/>
+      <x:c r="K29" s="1"/>
+      <x:c r="L29" s="1"/>
+      <x:c r="M29" s="1"/>
+      <x:c r="N29" s="1"/>
+      <x:c r="O29" s="1"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="1"/>
@@ -20454,6 +20762,11 @@
       <x:c r="H30" s="1"/>
       <x:c r="I30" s="1"/>
       <x:c r="J30" s="1"/>
+      <x:c r="K30" s="1"/>
+      <x:c r="L30" s="1"/>
+      <x:c r="M30" s="1"/>
+      <x:c r="N30" s="1"/>
+      <x:c r="O30" s="1"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="1"/>
@@ -20466,6 +20779,11 @@
       <x:c r="H31" s="1"/>
       <x:c r="I31" s="1"/>
       <x:c r="J31" s="1"/>
+      <x:c r="K31" s="1"/>
+      <x:c r="L31" s="1"/>
+      <x:c r="M31" s="1"/>
+      <x:c r="N31" s="1"/>
+      <x:c r="O31" s="1"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="1"/>
@@ -20478,6 +20796,11 @@
       <x:c r="H32" s="1"/>
       <x:c r="I32" s="1"/>
       <x:c r="J32" s="1"/>
+      <x:c r="K32" s="1"/>
+      <x:c r="L32" s="1"/>
+      <x:c r="M32" s="1"/>
+      <x:c r="N32" s="1"/>
+      <x:c r="O32" s="1"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="1"/>
@@ -20490,6 +20813,11 @@
       <x:c r="H33" s="1"/>
       <x:c r="I33" s="1"/>
       <x:c r="J33" s="1"/>
+      <x:c r="K33" s="1"/>
+      <x:c r="L33" s="1"/>
+      <x:c r="M33" s="1"/>
+      <x:c r="N33" s="1"/>
+      <x:c r="O33" s="1"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="1"/>
@@ -20502,6 +20830,11 @@
       <x:c r="H34" s="1"/>
       <x:c r="I34" s="1"/>
       <x:c r="J34" s="1"/>
+      <x:c r="K34" s="1"/>
+      <x:c r="L34" s="1"/>
+      <x:c r="M34" s="1"/>
+      <x:c r="N34" s="1"/>
+      <x:c r="O34" s="1"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="1"/>
@@ -20514,6 +20847,11 @@
       <x:c r="H35" s="1"/>
       <x:c r="I35" s="1"/>
       <x:c r="J35" s="1"/>
+      <x:c r="K35" s="1"/>
+      <x:c r="L35" s="1"/>
+      <x:c r="M35" s="1"/>
+      <x:c r="N35" s="1"/>
+      <x:c r="O35" s="1"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="1"/>
@@ -20526,6 +20864,11 @@
       <x:c r="H36" s="1"/>
       <x:c r="I36" s="1"/>
       <x:c r="J36" s="1"/>
+      <x:c r="K36" s="1"/>
+      <x:c r="L36" s="1"/>
+      <x:c r="M36" s="1"/>
+      <x:c r="N36" s="1"/>
+      <x:c r="O36" s="1"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="1"/>
@@ -20538,6 +20881,11 @@
       <x:c r="H37" s="1"/>
       <x:c r="I37" s="1"/>
       <x:c r="J37" s="1"/>
+      <x:c r="K37" s="1"/>
+      <x:c r="L37" s="1"/>
+      <x:c r="M37" s="1"/>
+      <x:c r="N37" s="1"/>
+      <x:c r="O37" s="1"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="1"/>
@@ -20550,6 +20898,11 @@
       <x:c r="H38" s="1"/>
       <x:c r="I38" s="1"/>
       <x:c r="J38" s="1"/>
+      <x:c r="K38" s="1"/>
+      <x:c r="L38" s="1"/>
+      <x:c r="M38" s="1"/>
+      <x:c r="N38" s="1"/>
+      <x:c r="O38" s="1"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="1"/>
@@ -20562,6 +20915,11 @@
       <x:c r="H39" s="1"/>
       <x:c r="I39" s="1"/>
       <x:c r="J39" s="1"/>
+      <x:c r="K39" s="1"/>
+      <x:c r="L39" s="1"/>
+      <x:c r="M39" s="1"/>
+      <x:c r="N39" s="1"/>
+      <x:c r="O39" s="1"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="1"/>
@@ -20574,6 +20932,11 @@
       <x:c r="H40" s="1"/>
       <x:c r="I40" s="1"/>
       <x:c r="J40" s="1"/>
+      <x:c r="K40" s="1"/>
+      <x:c r="L40" s="1"/>
+      <x:c r="M40" s="1"/>
+      <x:c r="N40" s="1"/>
+      <x:c r="O40" s="1"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="1"/>
@@ -20586,6 +20949,11 @@
       <x:c r="H41" s="1"/>
       <x:c r="I41" s="1"/>
       <x:c r="J41" s="1"/>
+      <x:c r="K41" s="1"/>
+      <x:c r="L41" s="1"/>
+      <x:c r="M41" s="1"/>
+      <x:c r="N41" s="1"/>
+      <x:c r="O41" s="1"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="1"/>
@@ -20598,6 +20966,11 @@
       <x:c r="H42" s="1"/>
       <x:c r="I42" s="1"/>
       <x:c r="J42" s="1"/>
+      <x:c r="K42" s="1"/>
+      <x:c r="L42" s="1"/>
+      <x:c r="M42" s="1"/>
+      <x:c r="N42" s="1"/>
+      <x:c r="O42" s="1"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="1"/>
@@ -20610,6 +20983,11 @@
       <x:c r="H43" s="1"/>
       <x:c r="I43" s="1"/>
       <x:c r="J43" s="1"/>
+      <x:c r="K43" s="1"/>
+      <x:c r="L43" s="1"/>
+      <x:c r="M43" s="1"/>
+      <x:c r="N43" s="1"/>
+      <x:c r="O43" s="1"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="1"/>
@@ -20622,6 +21000,11 @@
       <x:c r="H44" s="1"/>
       <x:c r="I44" s="1"/>
       <x:c r="J44" s="1"/>
+      <x:c r="K44" s="1"/>
+      <x:c r="L44" s="1"/>
+      <x:c r="M44" s="1"/>
+      <x:c r="N44" s="1"/>
+      <x:c r="O44" s="1"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="1"/>
@@ -20634,6 +21017,11 @@
       <x:c r="H45" s="1"/>
       <x:c r="I45" s="1"/>
       <x:c r="J45" s="1"/>
+      <x:c r="K45" s="1"/>
+      <x:c r="L45" s="1"/>
+      <x:c r="M45" s="1"/>
+      <x:c r="N45" s="1"/>
+      <x:c r="O45" s="1"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="1"/>
@@ -20646,6 +21034,11 @@
       <x:c r="H46" s="1"/>
       <x:c r="I46" s="1"/>
       <x:c r="J46" s="1"/>
+      <x:c r="K46" s="1"/>
+      <x:c r="L46" s="1"/>
+      <x:c r="M46" s="1"/>
+      <x:c r="N46" s="1"/>
+      <x:c r="O46" s="1"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="1"/>
@@ -20658,6 +21051,11 @@
       <x:c r="H47" s="1"/>
       <x:c r="I47" s="1"/>
       <x:c r="J47" s="1"/>
+      <x:c r="K47" s="1"/>
+      <x:c r="L47" s="1"/>
+      <x:c r="M47" s="1"/>
+      <x:c r="N47" s="1"/>
+      <x:c r="O47" s="1"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="1"/>
@@ -20670,6 +21068,11 @@
       <x:c r="H48" s="1"/>
       <x:c r="I48" s="1"/>
       <x:c r="J48" s="1"/>
+      <x:c r="K48" s="1"/>
+      <x:c r="L48" s="1"/>
+      <x:c r="M48" s="1"/>
+      <x:c r="N48" s="1"/>
+      <x:c r="O48" s="1"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="1"/>
@@ -20682,6 +21085,11 @@
       <x:c r="H49" s="1"/>
       <x:c r="I49" s="1"/>
       <x:c r="J49" s="1"/>
+      <x:c r="K49" s="1"/>
+      <x:c r="L49" s="1"/>
+      <x:c r="M49" s="1"/>
+      <x:c r="N49" s="1"/>
+      <x:c r="O49" s="1"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="1"/>
@@ -20694,6 +21102,11 @@
       <x:c r="H50" s="1"/>
       <x:c r="I50" s="1"/>
       <x:c r="J50" s="1"/>
+      <x:c r="K50" s="1"/>
+      <x:c r="L50" s="1"/>
+      <x:c r="M50" s="1"/>
+      <x:c r="N50" s="1"/>
+      <x:c r="O50" s="1"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="1"/>
@@ -20706,6 +21119,11 @@
       <x:c r="H51" s="1"/>
       <x:c r="I51" s="1"/>
       <x:c r="J51" s="1"/>
+      <x:c r="K51" s="1"/>
+      <x:c r="L51" s="1"/>
+      <x:c r="M51" s="1"/>
+      <x:c r="N51" s="1"/>
+      <x:c r="O51" s="1"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="1"/>
@@ -20718,6 +21136,11 @@
       <x:c r="H52" s="1"/>
       <x:c r="I52" s="1"/>
       <x:c r="J52" s="1"/>
+      <x:c r="K52" s="1"/>
+      <x:c r="L52" s="1"/>
+      <x:c r="M52" s="1"/>
+      <x:c r="N52" s="1"/>
+      <x:c r="O52" s="1"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="1"/>
@@ -20730,6 +21153,11 @@
       <x:c r="H53" s="1"/>
       <x:c r="I53" s="1"/>
       <x:c r="J53" s="1"/>
+      <x:c r="K53" s="1"/>
+      <x:c r="L53" s="1"/>
+      <x:c r="M53" s="1"/>
+      <x:c r="N53" s="1"/>
+      <x:c r="O53" s="1"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="1"/>
@@ -20742,6 +21170,11 @@
       <x:c r="H54" s="1"/>
       <x:c r="I54" s="1"/>
       <x:c r="J54" s="1"/>
+      <x:c r="K54" s="1"/>
+      <x:c r="L54" s="1"/>
+      <x:c r="M54" s="1"/>
+      <x:c r="N54" s="1"/>
+      <x:c r="O54" s="1"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="1"/>
@@ -20754,6 +21187,11 @@
       <x:c r="H55" s="1"/>
       <x:c r="I55" s="1"/>
       <x:c r="J55" s="1"/>
+      <x:c r="K55" s="1"/>
+      <x:c r="L55" s="1"/>
+      <x:c r="M55" s="1"/>
+      <x:c r="N55" s="1"/>
+      <x:c r="O55" s="1"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="1"/>
@@ -20766,6 +21204,11 @@
       <x:c r="H56" s="1"/>
       <x:c r="I56" s="1"/>
       <x:c r="J56" s="1"/>
+      <x:c r="K56" s="1"/>
+      <x:c r="L56" s="1"/>
+      <x:c r="M56" s="1"/>
+      <x:c r="N56" s="1"/>
+      <x:c r="O56" s="1"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="1"/>
@@ -20778,6 +21221,11 @@
       <x:c r="H57" s="1"/>
       <x:c r="I57" s="1"/>
       <x:c r="J57" s="1"/>
+      <x:c r="K57" s="1"/>
+      <x:c r="L57" s="1"/>
+      <x:c r="M57" s="1"/>
+      <x:c r="N57" s="1"/>
+      <x:c r="O57" s="1"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="1"/>
@@ -20790,6 +21238,11 @@
       <x:c r="H58" s="1"/>
       <x:c r="I58" s="1"/>
       <x:c r="J58" s="1"/>
+      <x:c r="K58" s="1"/>
+      <x:c r="L58" s="1"/>
+      <x:c r="M58" s="1"/>
+      <x:c r="N58" s="1"/>
+      <x:c r="O58" s="1"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="1"/>
@@ -20802,6 +21255,11 @@
       <x:c r="H59" s="1"/>
       <x:c r="I59" s="1"/>
       <x:c r="J59" s="1"/>
+      <x:c r="K59" s="1"/>
+      <x:c r="L59" s="1"/>
+      <x:c r="M59" s="1"/>
+      <x:c r="N59" s="1"/>
+      <x:c r="O59" s="1"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="1"/>
@@ -20814,6 +21272,11 @@
       <x:c r="H60" s="1"/>
       <x:c r="I60" s="1"/>
       <x:c r="J60" s="1"/>
+      <x:c r="K60" s="1"/>
+      <x:c r="L60" s="1"/>
+      <x:c r="M60" s="1"/>
+      <x:c r="N60" s="1"/>
+      <x:c r="O60" s="1"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="1"/>
@@ -20826,6 +21289,11 @@
       <x:c r="H61" s="1"/>
       <x:c r="I61" s="1"/>
       <x:c r="J61" s="1"/>
+      <x:c r="K61" s="1"/>
+      <x:c r="L61" s="1"/>
+      <x:c r="M61" s="1"/>
+      <x:c r="N61" s="1"/>
+      <x:c r="O61" s="1"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="1"/>
@@ -20838,6 +21306,11 @@
       <x:c r="H62" s="1"/>
       <x:c r="I62" s="1"/>
       <x:c r="J62" s="1"/>
+      <x:c r="K62" s="1"/>
+      <x:c r="L62" s="1"/>
+      <x:c r="M62" s="1"/>
+      <x:c r="N62" s="1"/>
+      <x:c r="O62" s="1"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="1"/>
@@ -20850,6 +21323,11 @@
       <x:c r="H63" s="1"/>
       <x:c r="I63" s="1"/>
       <x:c r="J63" s="1"/>
+      <x:c r="K63" s="1"/>
+      <x:c r="L63" s="1"/>
+      <x:c r="M63" s="1"/>
+      <x:c r="N63" s="1"/>
+      <x:c r="O63" s="1"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="1"/>
@@ -20862,6 +21340,11 @@
       <x:c r="H64" s="1"/>
       <x:c r="I64" s="1"/>
       <x:c r="J64" s="1"/>
+      <x:c r="K64" s="1"/>
+      <x:c r="L64" s="1"/>
+      <x:c r="M64" s="1"/>
+      <x:c r="N64" s="1"/>
+      <x:c r="O64" s="1"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="1"/>
@@ -20874,6 +21357,11 @@
       <x:c r="H65" s="1"/>
       <x:c r="I65" s="1"/>
       <x:c r="J65" s="1"/>
+      <x:c r="K65" s="1"/>
+      <x:c r="L65" s="1"/>
+      <x:c r="M65" s="1"/>
+      <x:c r="N65" s="1"/>
+      <x:c r="O65" s="1"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="1"/>
@@ -20886,6 +21374,11 @@
       <x:c r="H66" s="1"/>
       <x:c r="I66" s="1"/>
       <x:c r="J66" s="1"/>
+      <x:c r="K66" s="1"/>
+      <x:c r="L66" s="1"/>
+      <x:c r="M66" s="1"/>
+      <x:c r="N66" s="1"/>
+      <x:c r="O66" s="1"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="1"/>
@@ -20898,6 +21391,11 @@
       <x:c r="H67" s="1"/>
       <x:c r="I67" s="1"/>
       <x:c r="J67" s="1"/>
+      <x:c r="K67" s="1"/>
+      <x:c r="L67" s="1"/>
+      <x:c r="M67" s="1"/>
+      <x:c r="N67" s="1"/>
+      <x:c r="O67" s="1"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="1"/>
@@ -20910,6 +21408,11 @@
       <x:c r="H68" s="1"/>
       <x:c r="I68" s="1"/>
       <x:c r="J68" s="1"/>
+      <x:c r="K68" s="1"/>
+      <x:c r="L68" s="1"/>
+      <x:c r="M68" s="1"/>
+      <x:c r="N68" s="1"/>
+      <x:c r="O68" s="1"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="1"/>
@@ -20922,6 +21425,11 @@
       <x:c r="H69" s="1"/>
       <x:c r="I69" s="1"/>
       <x:c r="J69" s="1"/>
+      <x:c r="K69" s="1"/>
+      <x:c r="L69" s="1"/>
+      <x:c r="M69" s="1"/>
+      <x:c r="N69" s="1"/>
+      <x:c r="O69" s="1"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="1"/>
@@ -20934,6 +21442,11 @@
       <x:c r="H70" s="1"/>
       <x:c r="I70" s="1"/>
       <x:c r="J70" s="1"/>
+      <x:c r="K70" s="1"/>
+      <x:c r="L70" s="1"/>
+      <x:c r="M70" s="1"/>
+      <x:c r="N70" s="1"/>
+      <x:c r="O70" s="1"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="1"/>
@@ -20946,6 +21459,11 @@
       <x:c r="H71" s="1"/>
       <x:c r="I71" s="1"/>
       <x:c r="J71" s="1"/>
+      <x:c r="K71" s="1"/>
+      <x:c r="L71" s="1"/>
+      <x:c r="M71" s="1"/>
+      <x:c r="N71" s="1"/>
+      <x:c r="O71" s="1"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="1"/>
@@ -20958,6 +21476,11 @@
       <x:c r="H72" s="1"/>
       <x:c r="I72" s="1"/>
       <x:c r="J72" s="1"/>
+      <x:c r="K72" s="1"/>
+      <x:c r="L72" s="1"/>
+      <x:c r="M72" s="1"/>
+      <x:c r="N72" s="1"/>
+      <x:c r="O72" s="1"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="1"/>
@@ -20970,6 +21493,11 @@
       <x:c r="H73" s="1"/>
       <x:c r="I73" s="1"/>
       <x:c r="J73" s="1"/>
+      <x:c r="K73" s="1"/>
+      <x:c r="L73" s="1"/>
+      <x:c r="M73" s="1"/>
+      <x:c r="N73" s="1"/>
+      <x:c r="O73" s="1"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="1"/>
@@ -20982,6 +21510,11 @@
       <x:c r="H74" s="1"/>
       <x:c r="I74" s="1"/>
       <x:c r="J74" s="1"/>
+      <x:c r="K74" s="1"/>
+      <x:c r="L74" s="1"/>
+      <x:c r="M74" s="1"/>
+      <x:c r="N74" s="1"/>
+      <x:c r="O74" s="1"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="1"/>
@@ -20994,6 +21527,11 @@
       <x:c r="H75" s="1"/>
       <x:c r="I75" s="1"/>
       <x:c r="J75" s="1"/>
+      <x:c r="K75" s="1"/>
+      <x:c r="L75" s="1"/>
+      <x:c r="M75" s="1"/>
+      <x:c r="N75" s="1"/>
+      <x:c r="O75" s="1"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="1"/>
@@ -21006,6 +21544,11 @@
       <x:c r="H76" s="1"/>
       <x:c r="I76" s="1"/>
       <x:c r="J76" s="1"/>
+      <x:c r="K76" s="1"/>
+      <x:c r="L76" s="1"/>
+      <x:c r="M76" s="1"/>
+      <x:c r="N76" s="1"/>
+      <x:c r="O76" s="1"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="1"/>
@@ -21018,6 +21561,11 @@
       <x:c r="H77" s="1"/>
       <x:c r="I77" s="1"/>
       <x:c r="J77" s="1"/>
+      <x:c r="K77" s="1"/>
+      <x:c r="L77" s="1"/>
+      <x:c r="M77" s="1"/>
+      <x:c r="N77" s="1"/>
+      <x:c r="O77" s="1"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="1"/>
@@ -21030,6 +21578,11 @@
       <x:c r="H78" s="1"/>
       <x:c r="I78" s="1"/>
       <x:c r="J78" s="1"/>
+      <x:c r="K78" s="1"/>
+      <x:c r="L78" s="1"/>
+      <x:c r="M78" s="1"/>
+      <x:c r="N78" s="1"/>
+      <x:c r="O78" s="1"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="1"/>
@@ -21042,6 +21595,11 @@
       <x:c r="H79" s="1"/>
       <x:c r="I79" s="1"/>
       <x:c r="J79" s="1"/>
+      <x:c r="K79" s="1"/>
+      <x:c r="L79" s="1"/>
+      <x:c r="M79" s="1"/>
+      <x:c r="N79" s="1"/>
+      <x:c r="O79" s="1"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="1"/>
@@ -21054,16 +21612,25 @@
       <x:c r="H80" s="1"/>
       <x:c r="I80" s="1"/>
       <x:c r="J80" s="1"/>
+      <x:c r="K80" s="1"/>
+      <x:c r="L80" s="1"/>
+      <x:c r="M80" s="1"/>
+      <x:c r="N80" s="1"/>
+      <x:c r="O80" s="1"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:J1"/>
-    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L2"/>
     <x:mergeCell ref="A4:B4"/>
     <x:mergeCell ref="E4:F4"/>
+    <x:mergeCell ref="I4:J4"/>
+    <x:mergeCell ref="K4:L4"/>
+    <x:mergeCell ref="I5:J5"/>
+    <x:mergeCell ref="K5:L5"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00d66583a23d448d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21b4aebcef4941b2"/>
 </x:worksheet>
 </file>
 
@@ -21200,7 +21767,7 @@
         <x:f>B8+C8</x:f>
         <x:v>-1500</x:v>
       </x:c>
-      <x:c r="E8" s="69" t="n">
+      <x:c r="E8" s="87" t="n">
         <x:f>ABS(D8)/Assumptions!$B$10</x:f>
         <x:v>0.06666666666666667</x:v>
       </x:c>
@@ -21235,7 +21802,7 @@
         <x:f>B9+C9</x:f>
         <x:v>-6000</x:v>
       </x:c>
-      <x:c r="E9" s="69" t="n">
+      <x:c r="E9" s="87" t="n">
         <x:f>ABS(D9)/Assumptions!$B$10</x:f>
         <x:v>0.26666666666666666</x:v>
       </x:c>
@@ -21332,147 +21899,147 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="32" customHeight="1">
-      <x:c r="A15" s="70" t="str">
+      <x:c r="A15" s="88" t="str">
         <x:v>IRRBB_DV01</x:v>
       </x:c>
-      <x:c r="B15" s="70" t="str">
+      <x:c r="B15" s="88" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="C15" s="70" t="str">
+      <x:c r="C15" s="88" t="str">
         <x:v>plain_vanilla_interest_rate_swap</x:v>
       </x:c>
-      <x:c r="D15" s="70" t="str">
+      <x:c r="D15" s="88" t="str">
         <x:v>PAY_FIXED_RECEIVE_FLOAT</x:v>
       </x:c>
-      <x:c r="E15" s="71" t="n">
+      <x:c r="E15" s="89" t="n">
         <x:v>438.50875</x:v>
       </x:c>
-      <x:c r="F15" s="71" t="n">
+      <x:c r="F15" s="89" t="n">
         <x:v>-0.350807</x:v>
       </x:c>
-      <x:c r="G15" s="71" t="n">
+      <x:c r="G15" s="89" t="n">
         <x:v>-0.175404</x:v>
       </x:c>
-      <x:c r="H15" s="71" t="n">
+      <x:c r="H15" s="89" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="I15" s="72" t="str">
+      <x:c r="I15" s="90" t="str">
         <x:v>ALCO_REVIEW_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="32" customHeight="1">
-      <x:c r="A16" s="70" t="str">
+      <x:c r="A16" s="88" t="str">
         <x:v>IRRBB_DV01</x:v>
       </x:c>
-      <x:c r="B16" s="70" t="str">
+      <x:c r="B16" s="88" t="str">
         <x:v>TRY</x:v>
       </x:c>
-      <x:c r="C16" s="70" t="str">
+      <x:c r="C16" s="88" t="str">
         <x:v>plain_vanilla_interest_rate_swap</x:v>
       </x:c>
-      <x:c r="D16" s="70" t="str">
+      <x:c r="D16" s="88" t="str">
         <x:v>PAY_FIXED_RECEIVE_FLOAT</x:v>
       </x:c>
-      <x:c r="E16" s="71" t="n">
+      <x:c r="E16" s="89" t="n">
         <x:v>10316.64625</x:v>
       </x:c>
-      <x:c r="F16" s="71" t="n">
+      <x:c r="F16" s="89" t="n">
         <x:v>-8.253317</x:v>
       </x:c>
-      <x:c r="G16" s="71" t="n">
+      <x:c r="G16" s="89" t="n">
         <x:v>-4.126658</x:v>
       </x:c>
-      <x:c r="H16" s="71" t="n">
+      <x:c r="H16" s="89" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="I16" s="72" t="str">
+      <x:c r="I16" s="90" t="str">
         <x:v>ALCO_REVIEW_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="32" customHeight="1">
-      <x:c r="A17" s="70" t="str">
+      <x:c r="A17" s="88" t="str">
         <x:v>IRRBB_DV01</x:v>
       </x:c>
-      <x:c r="B17" s="70" t="str">
+      <x:c r="B17" s="88" t="str">
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="C17" s="70" t="str">
+      <x:c r="C17" s="88" t="str">
         <x:v>plain_vanilla_interest_rate_swap</x:v>
       </x:c>
-      <x:c r="D17" s="70" t="str">
+      <x:c r="D17" s="88" t="str">
         <x:v>RECEIVE_FIXED_PAY_FLOAT</x:v>
       </x:c>
-      <x:c r="E17" s="71" t="n">
+      <x:c r="E17" s="89" t="n">
         <x:v>163.53</x:v>
       </x:c>
-      <x:c r="F17" s="71" t="n">
+      <x:c r="F17" s="89" t="n">
         <x:v>0.130824</x:v>
       </x:c>
-      <x:c r="G17" s="71" t="n">
+      <x:c r="G17" s="89" t="n">
         <x:v>0.065412</x:v>
       </x:c>
-      <x:c r="H17" s="71" t="n">
+      <x:c r="H17" s="89" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="I17" s="72" t="str">
+      <x:c r="I17" s="90" t="str">
         <x:v>ALCO_REVIEW_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="32" customHeight="1">
-      <x:c r="A18" s="70" t="str">
+      <x:c r="A18" s="88" t="str">
         <x:v>FX_OPEN_POSITION</x:v>
       </x:c>
-      <x:c r="B18" s="70" t="str">
+      <x:c r="B18" s="88" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="C18" s="70" t="str">
+      <x:c r="C18" s="88" t="str">
         <x:v>fx_swap_or_forward</x:v>
       </x:c>
-      <x:c r="D18" s="70" t="str">
+      <x:c r="D18" s="88" t="str">
         <x:v>BUY_FX_SELL_TRY</x:v>
       </x:c>
-      <x:c r="E18" s="71" t="n">
+      <x:c r="E18" s="89" t="n">
         <x:v>1200</x:v>
       </x:c>
-      <x:c r="F18" s="71" t="n">
+      <x:c r="F18" s="89" t="n">
         <x:v>-1500</x:v>
       </x:c>
-      <x:c r="G18" s="71" t="n">
+      <x:c r="G18" s="89" t="n">
         <x:v>-300</x:v>
       </x:c>
-      <x:c r="H18" s="71" t="n">
+      <x:c r="H18" s="89" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="I18" s="72" t="str">
+      <x:c r="I18" s="90" t="str">
         <x:v>ALCO_REVIEW_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="32" customHeight="1">
-      <x:c r="A19" s="70" t="str">
+      <x:c r="A19" s="88" t="str">
         <x:v>FX_OPEN_POSITION</x:v>
       </x:c>
-      <x:c r="B19" s="70" t="str">
+      <x:c r="B19" s="88" t="str">
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="C19" s="70" t="str">
+      <x:c r="C19" s="88" t="str">
         <x:v>fx_swap_or_forward</x:v>
       </x:c>
-      <x:c r="D19" s="70" t="str">
+      <x:c r="D19" s="88" t="str">
         <x:v>BUY_FX_SELL_TRY</x:v>
       </x:c>
-      <x:c r="E19" s="71" t="n">
+      <x:c r="E19" s="89" t="n">
         <x:v>4800</x:v>
       </x:c>
-      <x:c r="F19" s="71" t="n">
+      <x:c r="F19" s="89" t="n">
         <x:v>-6000</x:v>
       </x:c>
-      <x:c r="G19" s="71" t="n">
+      <x:c r="G19" s="89" t="n">
         <x:v>-1200</x:v>
       </x:c>
-      <x:c r="H19" s="71" t="n">
+      <x:c r="H19" s="89" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="I19" s="72" t="str">
+      <x:c r="I19" s="90" t="str">
         <x:v>ALCO_REVIEW_REQUIRED</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat: add rapid digital-run liquidity stress scenario (#2)
Add a severe exploratory deposit-run scenario with front-loaded outflows, scenario-specific HQLA market-value shocks, a seven-day survival horizon, expanded validation, and refreshed ALCO deliverables.
</commit_message>
<xml_diff>
--- a/excel/Aurelia_Bank_ALCO_Risk_Workbench.xlsx
+++ b/excel/Aurelia_Bank_ALCO_Risk_Workbench.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="R7ca96f742fc34f50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R74d0fc161a134b02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="3" r:id="Re6c1f541f9a14706"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions Raw" sheetId="4" r:id="R11cb1113276b4f36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repricing Gap" sheetId="5" r:id="R8e08caf6c0174281"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IRRBB EVE" sheetId="6" r:id="R0c8d82c150484465"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NII Sensitivity" sheetId="7" r:id="R39c9b6df87744d80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liquidity" sheetId="8" r:id="Rbabadf0e8ff74114"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Hedge" sheetId="9" r:id="Rf9cf619124b34895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="10" r:id="R941d789cb3d0495e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="11" r:id="R523c953894234e0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="R2646fe77c57746d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R2c001d998e214b0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="3" r:id="R4c5f00fc29a74b55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions Raw" sheetId="4" r:id="Ra028822a1a274df8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repricing Gap" sheetId="5" r:id="Rbff1f6e00c114311"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IRRBB EVE" sheetId="6" r:id="R2f9c3bcd401d4451"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NII Sensitivity" sheetId="7" r:id="Re8498d649e104563"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liquidity" sheetId="8" r:id="R0b21fc60ca81473d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Hedge" sheetId="9" r:id="Rb3ef797d121c4a7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="10" r:id="R11249d17e03e4807"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="11" r:id="Re1f0334f7d5c4880"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,9 +20,9 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={9797CADA-ED84-CD56-90A0-55F03189A0F9}</x:author>
-    <x:author>tc={8B3D5F63-A3BE-10AA-5BD3-D8C17FABF35A}</x:author>
-    <x:author>tc={4A2F2257-0EC2-5C1F-0FC0-38DECE0247FF}</x:author>
+    <x:author>tc={C98EFE8F-088B-9606-9A45-E7FFDB6B4E80}</x:author>
+    <x:author>tc={270A24B8-4951-F9F8-1C31-B4A5E3B1C483}</x:author>
+    <x:author>tc={867C2A4C-7032-EFE8-6FE6-86305A326678}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B6" authorId="0">
@@ -221,7 +221,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="20">
+  <x:borders count="26">
     <x:border/>
     <x:border>
       <x:bottom style="double">
@@ -350,6 +350,48 @@
     </x:border>
     <x:border>
       <x:left style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:left>
+      <x:top style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:right>
+      <x:top style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:left>
+      <x:bottom style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:right>
+      <x:bottom style="medium">
+        <x:color rgb="FFC2413B"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="medium">
         <x:color rgb="FFC9D5DF"/>
       </x:left>
       <x:top style="medium">
@@ -394,7 +436,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="144">
+  <x:cellXfs count="162">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -482,6 +524,40 @@
     <x:xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="8" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="206" fontId="8" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="9" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="9" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="9" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="9" fillId="8" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="8" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="201" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -509,140 +585,140 @@
     <x:xf numFmtId="207" fontId="13" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="13" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="8" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="8" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="9" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="9" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="13" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="13" fillId="9" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="208" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1061,7 +1137,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>Combined stress takes LCR proxy below 100%</a:t>
+              <a:t>Rapid digital run exposes a seven-day survival horizon</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1080,7 +1156,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Executive Dashboard'!$H$19:$H$22</c:f>
+              <c:f>'Executive Dashboard'!$H$19:$H$23</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1088,7 +1164,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Executive Dashboard'!$I$19:$I$22</c:f>
+              <c:f>'Executive Dashboard'!$I$19:$I$23</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1443,7 +1519,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>LCR proxy under stress scenarios</a:t>
+              <a:t>Rapid digital run drives the LCR proxy to 78.1%</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1462,7 +1538,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Liquidity'!$L$8:$L$11</c:f>
+              <c:f>'Liquidity'!$N$8:$N$12</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1470,7 +1546,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Liquidity'!$M$8:$M$11</c:f>
+              <c:f>'Liquidity'!$O$8:$O$12</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1569,7 +1645,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R43ab1af045894983"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R366b5dbf276a4ca5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1599,7 +1675,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5c7b3c86ecce4fe7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R94bdfbe0b7ce4d2e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1634,7 +1710,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R05fd5df7c001460a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc7d492c98aeb41a2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1669,7 +1745,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0e213e15d56144dc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f91b34600324792"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1688,7 +1764,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1704,7 +1780,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R76806bd2dc7d4c13"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9ff97a2fcaf64970"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1715,7 +1791,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Murat Miraç Gedik" id="{A6D395B8-2D65-416B-B4C7-A973252CAC41}"/>
+  <xltc:person displayName="Murat Miraç Gedik" id="{6A530232-7AB4-4679-A611-99B52FBDEE6F}"/>
 </xltc:personList>
 </file>
 
@@ -1912,13 +1988,13 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B6" dT="2026-08-20T10:13:18.316" personId="{A6D395B8-2D65-416B-B4C7-A973252CAC41}" id="{9797CADA-ED84-CD56-90A0-55F03189A0F9}">
+  <xltc:threadedComment ref="B6" dT="2026-08-21T11:42:35.52" personId="{6A530232-7AB4-4679-A611-99B52FBDEE6F}" id="{C98EFE8F-088B-9606-9A45-E7FFDB6B4E80}">
     <xltc:text>Source: TCMB policy-rate announcement (2026 reference). https://www.tcmb.gov.tr/wps/wcm/connect/tr/tcmb+tr/main+menu/duyurular/basin/2026/duy2026-23</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B7" dT="2026-08-20T10:13:18.316" personId="{A6D395B8-2D65-416B-B4C7-A973252CAC41}" id="{8B3D5F63-A3BE-10AA-5BD3-D8C17FABF35A}">
+  <xltc:threadedComment ref="B7" dT="2026-08-21T11:42:35.52" personId="{6A530232-7AB4-4679-A611-99B52FBDEE6F}" id="{270A24B8-4951-F9F8-1C31-B4A5E3B1C483}">
     <xltc:text>Source: TCMB official exchange rates via e-Devlet, 2026-08-19. https://www.turkiye.gov.tr/doviz-kurlari</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="F6" dT="2026-08-20T10:13:18.316" personId="{A6D395B8-2D65-416B-B4C7-A973252CAC41}" id="{4A2F2257-0EC2-5C1F-0FC0-38DECE0247FF}">
+  <xltc:threadedComment ref="F6" dT="2026-08-21T11:42:35.52" personId="{6A530232-7AB4-4679-A611-99B52FBDEE6F}" id="{867C2A4C-7032-EFE8-6FE6-86305A326678}">
     <xltc:text>Source: Basel Committee, recalibration of IRRBB shocks (d578), effective 2026-01-01. https://www.bis.org/bcbs/publ/d578.pdf</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -1989,76 +2065,76 @@
       <x:c r="L3" s="1"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="78" t="str">
+      <x:c r="A4" s="96" t="str">
         <x:v>TOTAL ASSETS</x:v>
       </x:c>
-      <x:c r="B4" s="78"/>
-      <x:c r="C4" s="78" t="str">
+      <x:c r="B4" s="96"/>
+      <x:c r="C4" s="96" t="str">
         <x:v>WORST EVE LOSS</x:v>
       </x:c>
-      <x:c r="D4" s="78"/>
-      <x:c r="E4" s="78" t="str">
+      <x:c r="D4" s="96"/>
+      <x:c r="E4" s="96" t="str">
         <x:v>MAX |DELTA NII|</x:v>
       </x:c>
-      <x:c r="F4" s="78"/>
-      <x:c r="G4" s="78" t="str">
+      <x:c r="F4" s="96"/>
+      <x:c r="G4" s="96" t="str">
         <x:v>COMBINED LCR</x:v>
       </x:c>
-      <x:c r="H4" s="78"/>
-      <x:c r="I4" s="78" t="str">
+      <x:c r="H4" s="96"/>
+      <x:c r="I4" s="96" t="str">
         <x:v>FX OPEN / EQUITY</x:v>
       </x:c>
-      <x:c r="J4" s="78"/>
-      <x:c r="K4" s="78" t="str">
+      <x:c r="J4" s="96"/>
+      <x:c r="K4" s="96" t="str">
         <x:v>MODEL STATUS</x:v>
       </x:c>
-      <x:c r="L4" s="78"/>
+      <x:c r="L4" s="96"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="116" t="n">
+      <x:c r="A5" s="134" t="n">
         <x:f>'Balance Sheet'!F25</x:f>
         <x:v>180000</x:v>
       </x:c>
-      <x:c r="B5" s="117"/>
-      <x:c r="C5" s="126" t="n">
+      <x:c r="B5" s="135"/>
+      <x:c r="C5" s="144" t="n">
         <x:f>'IRRBB EVE'!C4</x:f>
         <x:v>0.13743893711111127</x:v>
       </x:c>
-      <x:c r="D5" s="126"/>
-      <x:c r="E5" s="118" t="n">
+      <x:c r="D5" s="144"/>
+      <x:c r="E5" s="136" t="n">
         <x:f>'NII Sensitivity'!C4</x:f>
         <x:v>0.058133649698356125</x:v>
       </x:c>
-      <x:c r="F5" s="118"/>
-      <x:c r="G5" s="128" t="n">
+      <x:c r="F5" s="136"/>
+      <x:c r="G5" s="146" t="n">
         <x:f>Liquidity!C4</x:f>
         <x:v>0.9483364199501884</x:v>
       </x:c>
-      <x:c r="H5" s="128"/>
-      <x:c r="I5" s="126" t="n">
+      <x:c r="H5" s="146"/>
+      <x:c r="I5" s="144" t="n">
         <x:f>'FX &amp; Hedge'!C4</x:f>
         <x:v>0.3333333333333333</x:v>
       </x:c>
-      <x:c r="J5" s="126"/>
-      <x:c r="K5" s="134" t="str">
+      <x:c r="J5" s="144"/>
+      <x:c r="K5" s="152" t="str">
         <x:f>Controls!F30</x:f>
         <x:v>OK - RISK FLAGS SURFACED</x:v>
       </x:c>
-      <x:c r="L5" s="135"/>
+      <x:c r="L5" s="153"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="121"/>
-      <x:c r="B6" s="122"/>
-      <x:c r="C6" s="127"/>
-      <x:c r="D6" s="127"/>
-      <x:c r="E6" s="123"/>
-      <x:c r="F6" s="123"/>
-      <x:c r="G6" s="129"/>
-      <x:c r="H6" s="129"/>
-      <x:c r="I6" s="127"/>
-      <x:c r="J6" s="127"/>
-      <x:c r="K6" s="136"/>
-      <x:c r="L6" s="137"/>
+      <x:c r="A6" s="139"/>
+      <x:c r="B6" s="140"/>
+      <x:c r="C6" s="145"/>
+      <x:c r="D6" s="145"/>
+      <x:c r="E6" s="141"/>
+      <x:c r="F6" s="141"/>
+      <x:c r="G6" s="147"/>
+      <x:c r="H6" s="147"/>
+      <x:c r="I6" s="145"/>
+      <x:c r="J6" s="145"/>
+      <x:c r="K6" s="154"/>
+      <x:c r="L6" s="155"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1"/>
@@ -2112,23 +2188,23 @@
         <x:v>ALCO interpretation</x:v>
       </x:c>
       <x:c r="G9" s="1"/>
-      <x:c r="H9" s="142" t="str">
+      <x:c r="H9" s="160" t="str">
         <x:v>1 | Approve an 80% FX hedge target: buy USD/EUR and sell TRY via FX swap or forward, subject to limits and execution controls.</x:v>
       </x:c>
-      <x:c r="I9" s="142"/>
-      <x:c r="J9" s="142"/>
-      <x:c r="K9" s="142"/>
-      <x:c r="L9" s="142"/>
+      <x:c r="I9" s="160"/>
+      <x:c r="J9" s="160"/>
+      <x:c r="K9" s="160"/>
+      <x:c r="L9" s="160"/>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="1" t="str">
         <x:v>EVE loss / Tier 1</x:v>
       </x:c>
-      <x:c r="B10" s="69" t="n">
+      <x:c r="B10" s="87" t="n">
         <x:f>'IRRBB EVE'!C4</x:f>
         <x:v>0.13743893711111127</x:v>
       </x:c>
-      <x:c r="C10" s="69" t="n">
+      <x:c r="C10" s="87" t="n">
         <x:f>Assumptions!B11</x:f>
         <x:v>0.15</x:v>
       </x:c>
@@ -2140,27 +2216,27 @@
         <x:f>IF(B10&lt;=C10,"WITHIN_LIMIT","BREACH")</x:f>
         <x:v>WITHIN_LIMIT</x:v>
       </x:c>
-      <x:c r="F10" s="70" t="str">
+      <x:c r="F10" s="88" t="str">
         <x:v>Parallel-up is the adverse EVE scenario</x:v>
       </x:c>
       <x:c r="G10" s="1"/>
-      <x:c r="H10" s="142" t="str">
+      <x:c r="H10" s="160" t="str">
         <x:v>2 | Preserve the liquidity buffer: combined-stress LCR proxy is 94.8% and survival reaches the 30-day floor.</x:v>
       </x:c>
-      <x:c r="I10" s="142"/>
-      <x:c r="J10" s="142"/>
-      <x:c r="K10" s="142"/>
-      <x:c r="L10" s="142"/>
+      <x:c r="I10" s="160"/>
+      <x:c r="J10" s="160"/>
+      <x:c r="K10" s="160"/>
+      <x:c r="L10" s="160"/>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
       <x:c r="A11" s="1" t="str">
         <x:v>Absolute Delta NII</x:v>
       </x:c>
-      <x:c r="B11" s="69" t="n">
+      <x:c r="B11" s="87" t="n">
         <x:f>'NII Sensitivity'!C4</x:f>
         <x:v>0.058133649698356125</x:v>
       </x:c>
-      <x:c r="C11" s="69" t="n">
+      <x:c r="C11" s="87" t="n">
         <x:f>Assumptions!B12</x:f>
         <x:v>0.12</x:v>
       </x:c>
@@ -2172,27 +2248,27 @@
         <x:f>IF(B11&lt;=C11,"WITHIN_LIMIT","BREACH")</x:f>
         <x:v>WITHIN_LIMIT</x:v>
       </x:c>
-      <x:c r="F11" s="70" t="str">
+      <x:c r="F11" s="88" t="str">
         <x:v>Parallel-down compresses 12-month NII</x:v>
       </x:c>
       <x:c r="G11" s="1"/>
-      <x:c r="H11" s="142" t="str">
-        <x:v>3 | Review TRY duration hedge sizing: indicative pay-fixed IRS notional is TRY 10.3bn for a 50% DV01 reduction.</x:v>
-      </x:c>
-      <x:c r="I11" s="142"/>
-      <x:c r="J11" s="142"/>
-      <x:c r="K11" s="142"/>
-      <x:c r="L11" s="142"/>
+      <x:c r="H11" s="160" t="str">
+        <x:v>3 | Activate rapid-run readiness: the exploratory LCR proxy is 78.1%, stressed HQLA loses TRY 1.46bn and survival falls to 7 days.</x:v>
+      </x:c>
+      <x:c r="I11" s="160"/>
+      <x:c r="J11" s="160"/>
+      <x:c r="K11" s="160"/>
+      <x:c r="L11" s="160"/>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
       <x:c r="A12" s="1" t="str">
         <x:v>Combined LCR proxy</x:v>
       </x:c>
-      <x:c r="B12" s="69" t="n">
+      <x:c r="B12" s="87" t="n">
         <x:f>Liquidity!C4</x:f>
         <x:v>0.9483364199501884</x:v>
       </x:c>
-      <x:c r="C12" s="69" t="n">
+      <x:c r="C12" s="87" t="n">
         <x:f>Assumptions!B13</x:f>
         <x:v>1</x:v>
       </x:c>
@@ -2204,31 +2280,31 @@
         <x:f>IF(B12&gt;=C12,"WITHIN_LIMIT","BREACH")</x:f>
         <x:v>BREACH</x:v>
       </x:c>
-      <x:c r="F12" s="70" t="str">
+      <x:c r="F12" s="88" t="str">
         <x:v>Buffer falls below 100% in combined stress</x:v>
       </x:c>
       <x:c r="G12" s="1"/>
-      <x:c r="H12" s="142" t="str">
-        <x:v>4 | Protect NII downside: calibrate deposit beta and repricing lags before changing product pricing or hedge mix.</x:v>
-      </x:c>
-      <x:c r="I12" s="142"/>
-      <x:c r="J12" s="142"/>
-      <x:c r="K12" s="142"/>
-      <x:c r="L12" s="142"/>
+      <x:c r="H12" s="160" t="str">
+        <x:v>4 | Review TRY duration hedge sizing: indicative pay-fixed IRS notional is TRY 10.3bn for a 50% DV01 reduction.</x:v>
+      </x:c>
+      <x:c r="I12" s="160"/>
+      <x:c r="J12" s="160"/>
+      <x:c r="K12" s="160"/>
+      <x:c r="L12" s="160"/>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
       <x:c r="A13" s="1" t="str">
         <x:v>Combined survival days</x:v>
       </x:c>
-      <x:c r="B13" s="138" t="n">
+      <x:c r="B13" s="156" t="n">
         <x:f>Liquidity!G4</x:f>
         <x:v>30</x:v>
       </x:c>
-      <x:c r="C13" s="138" t="n">
+      <x:c r="C13" s="156" t="n">
         <x:f>Assumptions!B15</x:f>
         <x:v>30</x:v>
       </x:c>
-      <x:c r="D13" s="139" t="n">
+      <x:c r="D13" s="157" t="n">
         <x:f>B13-C13</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -2236,27 +2312,27 @@
         <x:f>IF(B13&gt;=C13,"WITHIN_LIMIT","BREACH")</x:f>
         <x:v>WITHIN_LIMIT</x:v>
       </x:c>
-      <x:c r="F13" s="70" t="str">
+      <x:c r="F13" s="88" t="str">
         <x:v>Exactly at management floor</x:v>
       </x:c>
       <x:c r="G13" s="1"/>
-      <x:c r="H13" s="142" t="str">
-        <x:v>5 | Treat every hedge output as a decision-support recommendation; treasury execution remains outside the model.</x:v>
-      </x:c>
-      <x:c r="I13" s="142"/>
-      <x:c r="J13" s="142"/>
-      <x:c r="K13" s="142"/>
-      <x:c r="L13" s="142"/>
+      <x:c r="H13" s="160" t="str">
+        <x:v>5 | Protect NII downside and treat every hedge output as decision support; execution remains outside the model.</x:v>
+      </x:c>
+      <x:c r="I13" s="160"/>
+      <x:c r="J13" s="160"/>
+      <x:c r="K13" s="160"/>
+      <x:c r="L13" s="160"/>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
       <x:c r="A14" s="1" t="str">
         <x:v>FX open / equity</x:v>
       </x:c>
-      <x:c r="B14" s="69" t="n">
+      <x:c r="B14" s="87" t="n">
         <x:f>'FX &amp; Hedge'!C4</x:f>
         <x:v>0.3333333333333333</x:v>
       </x:c>
-      <x:c r="C14" s="69" t="n">
+      <x:c r="C14" s="87" t="n">
         <x:f>Assumptions!B16</x:f>
         <x:v>0.2</x:v>
       </x:c>
@@ -2268,15 +2344,15 @@
         <x:f>IF(B14&lt;=C14,"WITHIN_LIMIT","BREACH")</x:f>
         <x:v>BREACH</x:v>
       </x:c>
-      <x:c r="F14" s="70" t="str">
+      <x:c r="F14" s="88" t="str">
         <x:v>USD short is the dominant remediable breach</x:v>
       </x:c>
       <x:c r="G14" s="1"/>
-      <x:c r="H14" s="142"/>
-      <x:c r="I14" s="142"/>
-      <x:c r="J14" s="142"/>
-      <x:c r="K14" s="142"/>
-      <x:c r="L14" s="142"/>
+      <x:c r="H14" s="160"/>
+      <x:c r="I14" s="160"/>
+      <x:c r="J14" s="160"/>
+      <x:c r="K14" s="160"/>
+      <x:c r="L14" s="160"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1"/>
@@ -2355,11 +2431,11 @@
         <x:f>'IRRBB EVE'!H6</x:f>
         <x:v>parallel_up</x:v>
       </x:c>
-      <x:c r="B19" s="143" t="n">
+      <x:c r="B19" s="161" t="n">
         <x:f>'IRRBB EVE'!I6</x:f>
         <x:v>-3092.3760850000035</x:v>
       </x:c>
-      <x:c r="C19" s="69" t="n">
+      <x:c r="C19" s="87" t="n">
         <x:f>'IRRBB EVE'!J6</x:f>
         <x:v>-0.13743893711111127</x:v>
       </x:c>
@@ -2371,12 +2447,12 @@
         <x:f>Liquidity!A8</x:f>
         <x:v>base</x:v>
       </x:c>
-      <x:c r="I19" s="69" t="n">
-        <x:f>Liquidity!F8</x:f>
+      <x:c r="I19" s="87" t="n">
+        <x:f>Liquidity!H8</x:f>
         <x:v>1.5872167592988458</x:v>
       </x:c>
       <x:c r="J19" s="33" t="n">
-        <x:f>Liquidity!G8</x:f>
+        <x:f>Liquidity!I8</x:f>
         <x:v>365</x:v>
       </x:c>
       <x:c r="K19" s="1"/>
@@ -2387,11 +2463,11 @@
         <x:f>'IRRBB EVE'!H7</x:f>
         <x:v>parallel_down</x:v>
       </x:c>
-      <x:c r="B20" s="143" t="n">
+      <x:c r="B20" s="161" t="n">
         <x:f>'IRRBB EVE'!I7</x:f>
         <x:v>3658.5116899999994</x:v>
       </x:c>
-      <x:c r="C20" s="69" t="n">
+      <x:c r="C20" s="87" t="n">
         <x:f>'IRRBB EVE'!J7</x:f>
         <x:v>0.16260051955555552</x:v>
       </x:c>
@@ -2403,12 +2479,12 @@
         <x:f>Liquidity!A9</x:f>
         <x:v>idiosyncratic</x:v>
       </x:c>
-      <x:c r="I20" s="69" t="n">
-        <x:f>Liquidity!F9</x:f>
+      <x:c r="I20" s="87" t="n">
+        <x:f>Liquidity!H9</x:f>
         <x:v>1.2021857923497268</x:v>
       </x:c>
       <x:c r="J20" s="33" t="n">
-        <x:f>Liquidity!G9</x:f>
+        <x:f>Liquidity!I9</x:f>
         <x:v>365</x:v>
       </x:c>
       <x:c r="K20" s="1"/>
@@ -2419,11 +2495,11 @@
         <x:f>'IRRBB EVE'!H8</x:f>
         <x:v>steepener</x:v>
       </x:c>
-      <x:c r="B21" s="143" t="n">
+      <x:c r="B21" s="161" t="n">
         <x:f>'IRRBB EVE'!I8</x:f>
         <x:v>-574.5688130000053</x:v>
       </x:c>
-      <x:c r="C21" s="69" t="n">
+      <x:c r="C21" s="87" t="n">
         <x:f>'IRRBB EVE'!J8</x:f>
         <x:v>-0.025536391688889125</x:v>
       </x:c>
@@ -2435,12 +2511,12 @@
         <x:f>Liquidity!A10</x:f>
         <x:v>market_wide</x:v>
       </x:c>
-      <x:c r="I21" s="69" t="n">
-        <x:f>Liquidity!F10</x:f>
+      <x:c r="I21" s="87" t="n">
+        <x:f>Liquidity!H10</x:f>
         <x:v>1.380496420935205</x:v>
       </x:c>
       <x:c r="J21" s="33" t="n">
-        <x:f>Liquidity!G10</x:f>
+        <x:f>Liquidity!I10</x:f>
         <x:v>365</x:v>
       </x:c>
       <x:c r="K21" s="1"/>
@@ -2451,11 +2527,11 @@
         <x:f>'IRRBB EVE'!H9</x:f>
         <x:v>flattener</x:v>
       </x:c>
-      <x:c r="B22" s="143" t="n">
+      <x:c r="B22" s="161" t="n">
         <x:f>'IRRBB EVE'!I9</x:f>
         <x:v>-96.98068100000091</x:v>
       </x:c>
-      <x:c r="C22" s="69" t="n">
+      <x:c r="C22" s="87" t="n">
         <x:f>'IRRBB EVE'!J9</x:f>
         <x:v>-0.00431025248888893</x:v>
       </x:c>
@@ -2467,12 +2543,12 @@
         <x:f>Liquidity!A11</x:f>
         <x:v>combined</x:v>
       </x:c>
-      <x:c r="I22" s="69" t="n">
-        <x:f>Liquidity!F11</x:f>
+      <x:c r="I22" s="87" t="n">
+        <x:f>Liquidity!H11</x:f>
         <x:v>0.9483364199501884</x:v>
       </x:c>
       <x:c r="J22" s="33" t="n">
-        <x:f>Liquidity!G11</x:f>
+        <x:f>Liquidity!I11</x:f>
         <x:v>30</x:v>
       </x:c>
       <x:c r="K22" s="1"/>
@@ -2483,11 +2559,11 @@
         <x:f>'IRRBB EVE'!H10</x:f>
         <x:v>short_up</x:v>
       </x:c>
-      <x:c r="B23" s="143" t="n">
+      <x:c r="B23" s="161" t="n">
         <x:f>'IRRBB EVE'!I10</x:f>
         <x:v>-1362.5024140000023</x:v>
       </x:c>
-      <x:c r="C23" s="69" t="n">
+      <x:c r="C23" s="87" t="n">
         <x:f>'IRRBB EVE'!J10</x:f>
         <x:v>-0.060555662844444545</x:v>
       </x:c>
@@ -2495,9 +2571,18 @@
       <x:c r="E23" s="1"/>
       <x:c r="F23" s="1"/>
       <x:c r="G23" s="1"/>
-      <x:c r="H23" s="1"/>
-      <x:c r="I23" s="1"/>
-      <x:c r="J23" s="1"/>
+      <x:c r="H23" s="33" t="str">
+        <x:f>Liquidity!A12</x:f>
+        <x:v>rapid_digital_run</x:v>
+      </x:c>
+      <x:c r="I23" s="87" t="n">
+        <x:f>Liquidity!H12</x:f>
+        <x:v>0.7809151560078172</x:v>
+      </x:c>
+      <x:c r="J23" s="33" t="n">
+        <x:f>Liquidity!I12</x:f>
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="K23" s="1"/>
       <x:c r="L23" s="1"/>
     </x:row>
@@ -2506,11 +2591,11 @@
         <x:f>'IRRBB EVE'!H11</x:f>
         <x:v>short_down</x:v>
       </x:c>
-      <x:c r="B24" s="143" t="n">
+      <x:c r="B24" s="161" t="n">
         <x:f>'IRRBB EVE'!I11</x:f>
         <x:v>1462.7598829999988</x:v>
       </x:c>
-      <x:c r="C24" s="69" t="n">
+      <x:c r="C24" s="87" t="n">
         <x:f>'IRRBB EVE'!J11</x:f>
         <x:v>0.0650115503555555</x:v>
       </x:c>
@@ -3343,7 +3428,7 @@
     <x:cfRule type="containsText" dxfId="24" priority="5" operator="containsText" text="OK"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30022f37619347c8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R282e6f778e974f2d"/>
 </x:worksheet>
 </file>
 
@@ -4115,11 +4200,11 @@
         <x:v>Official/method sources</x:v>
       </x:c>
       <x:c r="B27" s="33" t="n">
-        <x:f>COUNTA(Sources!A5:A12)</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTA(Sources!A5:A13)</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C27" s="1" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D27" s="1" t="n">
         <x:f>B27-C27</x:f>
@@ -4190,18 +4275,18 @@
       <x:c r="M29" s="1"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="74" t="str">
+      <x:c r="A30" s="92" t="str">
         <x:v>MODEL STATUS</x:v>
       </x:c>
-      <x:c r="B30" s="75"/>
-      <x:c r="C30" s="75"/>
-      <x:c r="D30" s="75"/>
-      <x:c r="E30" s="75"/>
-      <x:c r="F30" s="75" t="str">
+      <x:c r="B30" s="93"/>
+      <x:c r="C30" s="93"/>
+      <x:c r="D30" s="93"/>
+      <x:c r="E30" s="93"/>
+      <x:c r="F30" s="93" t="str">
         <x:f>IF(COUNTIF(F21:F28,"FAIL")=0,"OK - RISK FLAGS SURFACED","REVIEW REQUIRED")</x:f>
         <x:v>OK - RISK FLAGS SURFACED</x:v>
       </x:c>
-      <x:c r="G30" s="76"/>
+      <x:c r="G30" s="94"/>
       <x:c r="H30" s="1"/>
       <x:c r="I30" s="1"/>
       <x:c r="J30" s="1"/>
@@ -5092,7 +5177,7 @@
       <x:c r="C5" s="1" t="str">
         <x:v>2026-01-01</x:v>
       </x:c>
-      <x:c r="D5" s="70" t="str">
+      <x:c r="D5" s="88" t="str">
         <x:v>TRY 400/500/300; USD 200/300/225; EUR 225/350/200</x:v>
       </x:c>
       <x:c r="E5" s="1" t="str">
@@ -5101,13 +5186,13 @@
       <x:c r="F5" s="1" t="str">
         <x:v>Basel Committee on Banking Supervision</x:v>
       </x:c>
-      <x:c r="G5" s="70" t="str">
+      <x:c r="G5" s="88" t="str">
         <x:v>https://www.bis.org/bcbs/publ/d578.pdf</x:v>
       </x:c>
-      <x:c r="H5" s="70" t="str">
+      <x:c r="H5" s="88" t="str">
         <x:v>official_methodology</x:v>
       </x:c>
-      <x:c r="I5" s="70" t="str">
+      <x:c r="I5" s="88" t="str">
         <x:v>Revised shocks implemented from 1 January 2026</x:v>
       </x:c>
     </x:row>
@@ -5121,7 +5206,7 @@
       <x:c r="C6" s="1" t="str">
         <x:v>current framework</x:v>
       </x:c>
-      <x:c r="D6" s="70" t="str">
+      <x:c r="D6" s="88" t="str">
         <x:v>HQLA / 30-day net cash outflows</x:v>
       </x:c>
       <x:c r="E6" s="1" t="str">
@@ -5130,13 +5215,13 @@
       <x:c r="F6" s="1" t="str">
         <x:v>Bank for International Settlements</x:v>
       </x:c>
-      <x:c r="G6" s="70" t="str">
+      <x:c r="G6" s="88" t="str">
         <x:v>https://www.bis.org/basel_framework/chapter/LCR/20.htm</x:v>
       </x:c>
-      <x:c r="H6" s="70" t="str">
+      <x:c r="H6" s="88" t="str">
         <x:v>official_methodology</x:v>
       </x:c>
-      <x:c r="I6" s="70" t="str">
+      <x:c r="I6" s="88" t="str">
         <x:v>Workbook output is labelled proxy, not a regulatory return</x:v>
       </x:c>
     </x:row>
@@ -5150,7 +5235,7 @@
       <x:c r="C7" s="1" t="str">
         <x:v>current framework</x:v>
       </x:c>
-      <x:c r="D7" s="70" t="str">
+      <x:c r="D7" s="88" t="str">
         <x:v>ASF / RSF</x:v>
       </x:c>
       <x:c r="E7" s="1" t="str">
@@ -5159,13 +5244,13 @@
       <x:c r="F7" s="1" t="str">
         <x:v>Bank for International Settlements</x:v>
       </x:c>
-      <x:c r="G7" s="70" t="str">
+      <x:c r="G7" s="88" t="str">
         <x:v>https://www.bis.org/basel_framework/chapter/NSF/20.htm</x:v>
       </x:c>
-      <x:c r="H7" s="70" t="str">
+      <x:c r="H7" s="88" t="str">
         <x:v>official_methodology</x:v>
       </x:c>
-      <x:c r="I7" s="70" t="str">
+      <x:c r="I7" s="88" t="str">
         <x:v>Workbook output is labelled proxy, not a regulatory return</x:v>
       </x:c>
     </x:row>
@@ -5179,7 +5264,7 @@
       <x:c r="C8" s="1" t="str">
         <x:v>2026-08-19</x:v>
       </x:c>
-      <x:c r="D8" s="70" t="n">
+      <x:c r="D8" s="88" t="n">
         <x:v>0.37</x:v>
       </x:c>
       <x:c r="E8" s="1" t="str">
@@ -5188,13 +5273,13 @@
       <x:c r="F8" s="1" t="str">
         <x:v>TCMB</x:v>
       </x:c>
-      <x:c r="G8" s="70" t="str">
+      <x:c r="G8" s="88" t="str">
         <x:v>https://www.tcmb.gov.tr/wps/wcm/connect/tr/tcmb+tr/main+menu/duyurular/basin/2026/duy2026-23</x:v>
       </x:c>
-      <x:c r="H8" s="70" t="str">
+      <x:c r="H8" s="88" t="str">
         <x:v>official_observation</x:v>
       </x:c>
-      <x:c r="I8" s="70" t="str">
+      <x:c r="I8" s="88" t="str">
         <x:v>Reference market context; not used as a bank position</x:v>
       </x:c>
     </x:row>
@@ -5208,7 +5293,7 @@
       <x:c r="C9" s="1" t="str">
         <x:v>2026-08-19</x:v>
       </x:c>
-      <x:c r="D9" s="70" t="n">
+      <x:c r="D9" s="88" t="n">
         <x:v>47.8467</x:v>
       </x:c>
       <x:c r="E9" s="1" t="str">
@@ -5217,13 +5302,13 @@
       <x:c r="F9" s="1" t="str">
         <x:v>TCMB via e-Devlet</x:v>
       </x:c>
-      <x:c r="G9" s="70" t="str">
+      <x:c r="G9" s="88" t="str">
         <x:v>https://www.turkiye.gov.tr/doviz-kurlari</x:v>
       </x:c>
-      <x:c r="H9" s="70" t="str">
+      <x:c r="H9" s="88" t="str">
         <x:v>official_observation</x:v>
       </x:c>
-      <x:c r="I9" s="70" t="str">
+      <x:c r="I9" s="88" t="str">
         <x:v>Public market observation</x:v>
       </x:c>
     </x:row>
@@ -5237,7 +5322,7 @@
       <x:c r="C10" s="1" t="str">
         <x:v>2026-08-19</x:v>
       </x:c>
-      <x:c r="D10" s="70" t="n">
+      <x:c r="D10" s="88" t="n">
         <x:v>55.5061</x:v>
       </x:c>
       <x:c r="E10" s="1" t="str">
@@ -5246,13 +5331,13 @@
       <x:c r="F10" s="1" t="str">
         <x:v>TCMB via e-Devlet</x:v>
       </x:c>
-      <x:c r="G10" s="70" t="str">
+      <x:c r="G10" s="88" t="str">
         <x:v>https://www.turkiye.gov.tr/doviz-kurlari</x:v>
       </x:c>
-      <x:c r="H10" s="70" t="str">
+      <x:c r="H10" s="88" t="str">
         <x:v>official_observation</x:v>
       </x:c>
-      <x:c r="I10" s="70" t="str">
+      <x:c r="I10" s="88" t="str">
         <x:v>Public market observation</x:v>
       </x:c>
     </x:row>
@@ -5266,7 +5351,7 @@
       <x:c r="C11" s="1" t="str">
         <x:v>2026-06-30</x:v>
       </x:c>
-      <x:c r="D11" s="70" t="str">
+      <x:c r="D11" s="88" t="str">
         <x:v>Assets 52,727,562; loans 26,791,320; deposits 30,109,453</x:v>
       </x:c>
       <x:c r="E11" s="1" t="str">
@@ -5275,13 +5360,13 @@
       <x:c r="F11" s="1" t="str">
         <x:v>BDDK</x:v>
       </x:c>
-      <x:c r="G11" s="70" t="str">
+      <x:c r="G11" s="88" t="str">
         <x:v>https://www.bddk.org.tr/BultenAylik/tr/Home/HaberBulteni</x:v>
       </x:c>
-      <x:c r="H11" s="70" t="str">
+      <x:c r="H11" s="88" t="str">
         <x:v>official_benchmark</x:v>
       </x:c>
-      <x:c r="I11" s="70" t="str">
+      <x:c r="I11" s="88" t="str">
         <x:v>Contextual benchmark only; Aurelia bank is fictional</x:v>
       </x:c>
     </x:row>
@@ -5295,7 +5380,7 @@
       <x:c r="C12" s="1" t="str">
         <x:v>2026-08-19</x:v>
       </x:c>
-      <x:c r="D12" s="70" t="str">
+      <x:c r="D12" s="88" t="str">
         <x:v>Deterministic seed 20260819</x:v>
       </x:c>
       <x:c r="E12" s="1" t="str">
@@ -5304,26 +5389,44 @@
       <x:c r="F12" s="1" t="str">
         <x:v>Project generator</x:v>
       </x:c>
-      <x:c r="G12" s="70" t="str">
+      <x:c r="G12" s="88" t="str">
         <x:v>docs/data_provenance.md</x:v>
       </x:c>
-      <x:c r="H12" s="70" t="str">
+      <x:c r="H12" s="88" t="str">
         <x:v>controlled_synthetic</x:v>
       </x:c>
-      <x:c r="I12" s="70" t="str">
+      <x:c r="I12" s="88" t="str">
         <x:v>No customer data, PII or confidential bank data</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="1"/>
-      <x:c r="B13" s="1"/>
-      <x:c r="C13" s="1"/>
-      <x:c r="D13" s="1"/>
-      <x:c r="E13" s="1"/>
-      <x:c r="F13" s="1"/>
-      <x:c r="G13" s="1"/>
-      <x:c r="H13" s="1"/>
-      <x:c r="I13" s="1"/>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="1" t="str">
+        <x:v>AURELIA-DIGITAL-RUN</x:v>
+      </x:c>
+      <x:c r="B13" s="1" t="str">
+        <x:v>Rapid digital deposit-run assumptions</x:v>
+      </x:c>
+      <x:c r="C13" s="1" t="str">
+        <x:v>2026-08-21</x:v>
+      </x:c>
+      <x:c r="D13" s="88" t="str">
+        <x:v>45% demand; 30% term; 55% day 1; 85% day 7</x:v>
+      </x:c>
+      <x:c r="E13" s="1" t="str">
+        <x:v>scenario parameters</x:v>
+      </x:c>
+      <x:c r="F13" s="1" t="str">
+        <x:v>Internal ALCO demonstration scenario</x:v>
+      </x:c>
+      <x:c r="G13" s="88" t="str">
+        <x:v>docs/rapid_digital_run_scenario.md</x:v>
+      </x:c>
+      <x:c r="H13" s="88" t="str">
+        <x:v>controlled_internal_assumption</x:v>
+      </x:c>
+      <x:c r="I13" s="88" t="str">
+        <x:v>Severe exploratory vulnerability test; not a forecast or regulatory calibration</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1"/>
@@ -7187,7 +7290,7 @@
     <x:mergeCell ref="E12:J12"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31f625cb559148df"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4522e2ee601d49ec"/>
 </x:worksheet>
 </file>
 
@@ -19046,7 +19149,7 @@
     <x:mergeCell ref="A4:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re583719015c5427a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40f6aec535884b7d"/>
 </x:worksheet>
 </file>
 
@@ -19911,7 +20014,7 @@
     <x:mergeCell ref="A4:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6664cecc1c2d41de"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55524bdc76794467"/>
 </x:worksheet>
 </file>
 
@@ -19919,16 +20022,18 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -19944,10 +20049,15 @@
       <x:c r="H1" s="4"/>
       <x:c r="I1" s="4"/>
       <x:c r="J1" s="4"/>
+      <x:c r="K1" s="4"/>
+      <x:c r="L1" s="4"/>
+      <x:c r="M1" s="1"/>
+      <x:c r="N1" s="1"/>
+      <x:c r="O1" s="1"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>LCR and NSFR proxy analytics for portfolio demonstration; not a regulatory return</x:v>
+        <x:v>Five governed management scenarios including a severe rapid digital run; not a regulatory return</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -19958,6 +20068,11 @@
       <x:c r="H2" s="7"/>
       <x:c r="I2" s="7"/>
       <x:c r="J2" s="7"/>
+      <x:c r="K2" s="7"/>
+      <x:c r="L2" s="7"/>
+      <x:c r="M2" s="1"/>
+      <x:c r="N2" s="1"/>
+      <x:c r="O2" s="1"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1"/>
@@ -19970,6 +20085,11 @@
       <x:c r="H3" s="1"/>
       <x:c r="I3" s="1"/>
       <x:c r="J3" s="1"/>
+      <x:c r="K3" s="1"/>
+      <x:c r="L3" s="1"/>
+      <x:c r="M3" s="1"/>
+      <x:c r="N3" s="1"/>
+      <x:c r="O3" s="1"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="61" t="str">
@@ -19977,7 +20097,7 @@
       </x:c>
       <x:c r="B4" s="62"/>
       <x:c r="C4" s="63" t="n">
-        <x:f>F11</x:f>
+        <x:f>H11</x:f>
         <x:v>0.9483364199501884</x:v>
       </x:c>
       <x:c r="D4" s="1"/>
@@ -19986,12 +20106,22 @@
       </x:c>
       <x:c r="F4" s="67"/>
       <x:c r="G4" s="68" t="n">
-        <x:f>G11</x:f>
+        <x:f>I11</x:f>
         <x:v>30</x:v>
       </x:c>
       <x:c r="H4" s="1"/>
-      <x:c r="I4" s="1"/>
-      <x:c r="J4" s="1"/>
+      <x:c r="I4" s="79" t="str">
+        <x:v>Rapid-run LCR proxy</x:v>
+      </x:c>
+      <x:c r="J4" s="80"/>
+      <x:c r="K4" s="81" t="n">
+        <x:f>H12</x:f>
+        <x:v>0.7809151560078172</x:v>
+      </x:c>
+      <x:c r="L4" s="82"/>
+      <x:c r="M4" s="1"/>
+      <x:c r="N4" s="1"/>
+      <x:c r="O4" s="1"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="1"/>
@@ -20002,8 +20132,18 @@
       <x:c r="F5" s="1"/>
       <x:c r="G5" s="1"/>
       <x:c r="H5" s="1"/>
-      <x:c r="I5" s="1"/>
-      <x:c r="J5" s="1"/>
+      <x:c r="I5" s="83" t="str">
+        <x:v>Rapid-run survival</x:v>
+      </x:c>
+      <x:c r="J5" s="84"/>
+      <x:c r="K5" s="85" t="n">
+        <x:f>I12</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="L5" s="86"/>
+      <x:c r="M5" s="1"/>
+      <x:c r="N5" s="1"/>
+      <x:c r="O5" s="1"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="1"/>
@@ -20016,42 +20156,54 @@
       <x:c r="H6" s="1"/>
       <x:c r="I6" s="1"/>
       <x:c r="J6" s="1"/>
+      <x:c r="K6" s="1"/>
+      <x:c r="L6" s="1"/>
+      <x:c r="M6" s="1"/>
+      <x:c r="N6" s="1"/>
+      <x:c r="O6" s="1"/>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="24" t="str">
         <x:v>Scenario</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>HQLA</x:v>
+        <x:v>Base HQLA</x:v>
       </x:c>
       <x:c r="C7" s="24" t="str">
+        <x:v>Stressed HQLA</x:v>
+      </x:c>
+      <x:c r="D7" s="24" t="str">
+        <x:v>HQLA MV loss</x:v>
+      </x:c>
+      <x:c r="E7" s="24" t="str">
         <x:v>Gross outflows 30d</x:v>
       </x:c>
-      <x:c r="D7" s="24" t="str">
+      <x:c r="F7" s="24" t="str">
         <x:v>Eligible inflows 30d</x:v>
       </x:c>
-      <x:c r="E7" s="24" t="str">
+      <x:c r="G7" s="24" t="str">
         <x:v>Net outflows 30d</x:v>
       </x:c>
-      <x:c r="F7" s="24" t="str">
+      <x:c r="H7" s="24" t="str">
         <x:v>LCR proxy</x:v>
       </x:c>
-      <x:c r="G7" s="24" t="str">
+      <x:c r="I7" s="24" t="str">
         <x:v>Survival days</x:v>
       </x:c>
-      <x:c r="H7" s="24" t="str">
+      <x:c r="J7" s="24" t="str">
         <x:v>ASF</x:v>
       </x:c>
-      <x:c r="I7" s="24" t="str">
+      <x:c r="K7" s="24" t="str">
         <x:v>RSF</x:v>
       </x:c>
-      <x:c r="J7" s="24" t="str">
+      <x:c r="L7" s="24" t="str">
         <x:v>NSFR proxy</x:v>
       </x:c>
-      <x:c r="L7" t="str">
+      <x:c r="M7" s="1"/>
+      <x:c r="N7" s="1" t="str">
         <x:v>Scenario</x:v>
       </x:c>
-      <x:c r="M7" t="str">
+      <x:c r="O7" s="1" t="str">
         <x:v>LCR proxy</x:v>
       </x:c>
     </x:row>
@@ -20063,38 +20215,46 @@
         <x:v>59400</x:v>
       </x:c>
       <x:c r="C8" s="13" t="n">
+        <x:v>59400</x:v>
+      </x:c>
+      <x:c r="D8" s="13" t="n">
+        <x:f>B8-C8</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="13" t="n">
         <x:v>37424</x:v>
       </x:c>
-      <x:c r="D8" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E8" s="13" t="n">
-        <x:f>C8-MIN(D8,C8*75%)</x:f>
+      <x:c r="F8" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="13" t="n">
+        <x:f>E8-MIN(F8,E8*75%)</x:f>
         <x:v>37424</x:v>
       </x:c>
-      <x:c r="F8" s="11" t="n">
-        <x:f>B8/E8</x:f>
+      <x:c r="H8" s="11" t="n">
+        <x:f>C8/G8</x:f>
         <x:v>1.5872167592988458</x:v>
       </x:c>
-      <x:c r="G8" s="1" t="n">
+      <x:c r="I8" s="1" t="n">
         <x:v>365</x:v>
       </x:c>
-      <x:c r="H8" s="13" t="n">
+      <x:c r="J8" s="13" t="n">
         <x:v>150450</x:v>
       </x:c>
-      <x:c r="I8" s="13" t="n">
+      <x:c r="K8" s="13" t="n">
         <x:v>104950</x:v>
       </x:c>
-      <x:c r="J8" s="11" t="n">
-        <x:f>H8/I8</x:f>
+      <x:c r="L8" s="11" t="n">
+        <x:f>J8/K8</x:f>
         <x:v>1.4335397808480228</x:v>
       </x:c>
-      <x:c r="L8" t="str">
+      <x:c r="M8" s="1"/>
+      <x:c r="N8" s="1" t="str">
         <x:f>A8</x:f>
         <x:v>base</x:v>
       </x:c>
-      <x:c r="M8" t="n">
-        <x:f>F8</x:f>
+      <x:c r="O8" s="1" t="n">
+        <x:f>H8</x:f>
         <x:v>1.5872167592988458</x:v>
       </x:c>
     </x:row>
@@ -20106,38 +20266,46 @@
         <x:v>59400</x:v>
       </x:c>
       <x:c r="C9" s="13" t="n">
+        <x:v>59400</x:v>
+      </x:c>
+      <x:c r="D9" s="13" t="n">
+        <x:f>B9-C9</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="13" t="n">
         <x:v>49410</x:v>
       </x:c>
-      <x:c r="D9" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E9" s="13" t="n">
-        <x:f>C9-MIN(D9,C9*75%)</x:f>
+      <x:c r="F9" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="13" t="n">
+        <x:f>E9-MIN(F9,E9*75%)</x:f>
         <x:v>49410</x:v>
       </x:c>
-      <x:c r="F9" s="11" t="n">
-        <x:f>B9/E9</x:f>
+      <x:c r="H9" s="11" t="n">
+        <x:f>C9/G9</x:f>
         <x:v>1.2021857923497268</x:v>
       </x:c>
-      <x:c r="G9" s="1" t="n">
+      <x:c r="I9" s="1" t="n">
         <x:v>365</x:v>
       </x:c>
-      <x:c r="H9" s="13" t="n">
+      <x:c r="J9" s="13" t="n">
         <x:v>150450</x:v>
       </x:c>
-      <x:c r="I9" s="13" t="n">
+      <x:c r="K9" s="13" t="n">
         <x:v>104950</x:v>
       </x:c>
-      <x:c r="J9" s="11" t="n">
-        <x:f>H9/I9</x:f>
+      <x:c r="L9" s="11" t="n">
+        <x:f>J9/K9</x:f>
         <x:v>1.4335397808480228</x:v>
       </x:c>
-      <x:c r="L9" t="str">
+      <x:c r="M9" s="1"/>
+      <x:c r="N9" s="1" t="str">
         <x:f>A9</x:f>
         <x:v>idiosyncratic</x:v>
       </x:c>
-      <x:c r="M9" t="n">
-        <x:f>F9</x:f>
+      <x:c r="O9" s="1" t="n">
+        <x:f>H9</x:f>
         <x:v>1.2021857923497268</x:v>
       </x:c>
     </x:row>
@@ -20149,38 +20317,46 @@
         <x:v>59400</x:v>
       </x:c>
       <x:c r="C10" s="13" t="n">
+        <x:v>59400</x:v>
+      </x:c>
+      <x:c r="D10" s="13" t="n">
+        <x:f>B10-C10</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="13" t="n">
         <x:v>43028</x:v>
       </x:c>
-      <x:c r="D10" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E10" s="13" t="n">
-        <x:f>C10-MIN(D10,C10*75%)</x:f>
+      <x:c r="F10" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" s="13" t="n">
+        <x:f>E10-MIN(F10,E10*75%)</x:f>
         <x:v>43028</x:v>
       </x:c>
-      <x:c r="F10" s="11" t="n">
-        <x:f>B10/E10</x:f>
+      <x:c r="H10" s="11" t="n">
+        <x:f>C10/G10</x:f>
         <x:v>1.380496420935205</x:v>
       </x:c>
-      <x:c r="G10" s="1" t="n">
+      <x:c r="I10" s="1" t="n">
         <x:v>365</x:v>
       </x:c>
-      <x:c r="H10" s="13" t="n">
+      <x:c r="J10" s="13" t="n">
         <x:v>150450</x:v>
       </x:c>
-      <x:c r="I10" s="13" t="n">
+      <x:c r="K10" s="13" t="n">
         <x:v>104950</x:v>
       </x:c>
-      <x:c r="J10" s="11" t="n">
-        <x:f>H10/I10</x:f>
+      <x:c r="L10" s="11" t="n">
+        <x:f>J10/K10</x:f>
         <x:v>1.4335397808480228</x:v>
       </x:c>
-      <x:c r="L10" t="str">
+      <x:c r="M10" s="1"/>
+      <x:c r="N10" s="1" t="str">
         <x:f>A10</x:f>
         <x:v>market_wide</x:v>
       </x:c>
-      <x:c r="M10" t="n">
-        <x:f>F10</x:f>
+      <x:c r="O10" s="1" t="n">
+        <x:f>H10</x:f>
         <x:v>1.380496420935205</x:v>
       </x:c>
     </x:row>
@@ -20192,52 +20368,99 @@
         <x:v>59400</x:v>
       </x:c>
       <x:c r="C11" s="13" t="n">
+        <x:v>59400</x:v>
+      </x:c>
+      <x:c r="D11" s="13" t="n">
+        <x:f>B11-C11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="13" t="n">
         <x:v>62636</x:v>
       </x:c>
-      <x:c r="D11" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E11" s="13" t="n">
-        <x:f>C11-MIN(D11,C11*75%)</x:f>
+      <x:c r="F11" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G11" s="13" t="n">
+        <x:f>E11-MIN(F11,E11*75%)</x:f>
         <x:v>62636</x:v>
       </x:c>
-      <x:c r="F11" s="11" t="n">
-        <x:f>B11/E11</x:f>
+      <x:c r="H11" s="11" t="n">
+        <x:f>C11/G11</x:f>
         <x:v>0.9483364199501884</x:v>
       </x:c>
-      <x:c r="G11" s="1" t="n">
+      <x:c r="I11" s="1" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="H11" s="13" t="n">
+      <x:c r="J11" s="13" t="n">
         <x:v>150450</x:v>
       </x:c>
-      <x:c r="I11" s="13" t="n">
+      <x:c r="K11" s="13" t="n">
         <x:v>104950</x:v>
       </x:c>
-      <x:c r="J11" s="11" t="n">
-        <x:f>H11/I11</x:f>
+      <x:c r="L11" s="11" t="n">
+        <x:f>J11/K11</x:f>
         <x:v>1.4335397808480228</x:v>
       </x:c>
-      <x:c r="L11" t="str">
+      <x:c r="M11" s="1"/>
+      <x:c r="N11" s="1" t="str">
         <x:f>A11</x:f>
         <x:v>combined</x:v>
       </x:c>
-      <x:c r="M11" t="n">
-        <x:f>F11</x:f>
+      <x:c r="O11" s="1" t="n">
+        <x:f>H11</x:f>
         <x:v>0.9483364199501884</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="1"/>
-      <x:c r="B12" s="1"/>
-      <x:c r="C12" s="1"/>
-      <x:c r="D12" s="1"/>
-      <x:c r="E12" s="1"/>
-      <x:c r="F12" s="1"/>
-      <x:c r="G12" s="1"/>
-      <x:c r="H12" s="1"/>
-      <x:c r="I12" s="1"/>
-      <x:c r="J12" s="1"/>
+      <x:c r="A12" s="1" t="str">
+        <x:v>rapid_digital_run</x:v>
+      </x:c>
+      <x:c r="B12" s="13" t="n">
+        <x:v>59400</x:v>
+      </x:c>
+      <x:c r="C12" s="13" t="n">
+        <x:v>57940</x:v>
+      </x:c>
+      <x:c r="D12" s="13" t="n">
+        <x:f>B12-C12</x:f>
+        <x:v>1460</x:v>
+      </x:c>
+      <x:c r="E12" s="13" t="n">
+        <x:v>74195</x:v>
+      </x:c>
+      <x:c r="F12" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" s="13" t="n">
+        <x:f>E12-MIN(F12,E12*75%)</x:f>
+        <x:v>74195</x:v>
+      </x:c>
+      <x:c r="H12" s="11" t="n">
+        <x:f>C12/G12</x:f>
+        <x:v>0.7809151560078172</x:v>
+      </x:c>
+      <x:c r="I12" s="1" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J12" s="13" t="n">
+        <x:v>150450</x:v>
+      </x:c>
+      <x:c r="K12" s="13" t="n">
+        <x:v>104950</x:v>
+      </x:c>
+      <x:c r="L12" s="11" t="n">
+        <x:f>J12/K12</x:f>
+        <x:v>1.4335397808480228</x:v>
+      </x:c>
+      <x:c r="M12" s="1"/>
+      <x:c r="N12" s="1" t="str">
+        <x:f>A12</x:f>
+        <x:v>rapid_digital_run</x:v>
+      </x:c>
+      <x:c r="O12" s="1" t="n">
+        <x:f>H12</x:f>
+        <x:v>0.7809151560078172</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1"/>
@@ -20250,6 +20473,11 @@
       <x:c r="H13" s="1"/>
       <x:c r="I13" s="1"/>
       <x:c r="J13" s="1"/>
+      <x:c r="K13" s="1"/>
+      <x:c r="L13" s="1"/>
+      <x:c r="M13" s="1"/>
+      <x:c r="N13" s="1"/>
+      <x:c r="O13" s="1"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1"/>
@@ -20262,6 +20490,11 @@
       <x:c r="H14" s="1"/>
       <x:c r="I14" s="1"/>
       <x:c r="J14" s="1"/>
+      <x:c r="K14" s="1"/>
+      <x:c r="L14" s="1"/>
+      <x:c r="M14" s="1"/>
+      <x:c r="N14" s="1"/>
+      <x:c r="O14" s="1"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1"/>
@@ -20274,6 +20507,11 @@
       <x:c r="H15" s="1"/>
       <x:c r="I15" s="1"/>
       <x:c r="J15" s="1"/>
+      <x:c r="K15" s="1"/>
+      <x:c r="L15" s="1"/>
+      <x:c r="M15" s="1"/>
+      <x:c r="N15" s="1"/>
+      <x:c r="O15" s="1"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1"/>
@@ -20286,6 +20524,11 @@
       <x:c r="H16" s="1"/>
       <x:c r="I16" s="1"/>
       <x:c r="J16" s="1"/>
+      <x:c r="K16" s="1"/>
+      <x:c r="L16" s="1"/>
+      <x:c r="M16" s="1"/>
+      <x:c r="N16" s="1"/>
+      <x:c r="O16" s="1"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="1"/>
@@ -20298,6 +20541,11 @@
       <x:c r="H17" s="1"/>
       <x:c r="I17" s="1"/>
       <x:c r="J17" s="1"/>
+      <x:c r="K17" s="1"/>
+      <x:c r="L17" s="1"/>
+      <x:c r="M17" s="1"/>
+      <x:c r="N17" s="1"/>
+      <x:c r="O17" s="1"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="1"/>
@@ -20310,6 +20558,11 @@
       <x:c r="H18" s="1"/>
       <x:c r="I18" s="1"/>
       <x:c r="J18" s="1"/>
+      <x:c r="K18" s="1"/>
+      <x:c r="L18" s="1"/>
+      <x:c r="M18" s="1"/>
+      <x:c r="N18" s="1"/>
+      <x:c r="O18" s="1"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="1"/>
@@ -20322,6 +20575,11 @@
       <x:c r="H19" s="1"/>
       <x:c r="I19" s="1"/>
       <x:c r="J19" s="1"/>
+      <x:c r="K19" s="1"/>
+      <x:c r="L19" s="1"/>
+      <x:c r="M19" s="1"/>
+      <x:c r="N19" s="1"/>
+      <x:c r="O19" s="1"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="1"/>
@@ -20334,6 +20592,11 @@
       <x:c r="H20" s="1"/>
       <x:c r="I20" s="1"/>
       <x:c r="J20" s="1"/>
+      <x:c r="K20" s="1"/>
+      <x:c r="L20" s="1"/>
+      <x:c r="M20" s="1"/>
+      <x:c r="N20" s="1"/>
+      <x:c r="O20" s="1"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="1"/>
@@ -20346,6 +20609,11 @@
       <x:c r="H21" s="1"/>
       <x:c r="I21" s="1"/>
       <x:c r="J21" s="1"/>
+      <x:c r="K21" s="1"/>
+      <x:c r="L21" s="1"/>
+      <x:c r="M21" s="1"/>
+      <x:c r="N21" s="1"/>
+      <x:c r="O21" s="1"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="1"/>
@@ -20358,6 +20626,11 @@
       <x:c r="H22" s="1"/>
       <x:c r="I22" s="1"/>
       <x:c r="J22" s="1"/>
+      <x:c r="K22" s="1"/>
+      <x:c r="L22" s="1"/>
+      <x:c r="M22" s="1"/>
+      <x:c r="N22" s="1"/>
+      <x:c r="O22" s="1"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="1"/>
@@ -20370,6 +20643,11 @@
       <x:c r="H23" s="1"/>
       <x:c r="I23" s="1"/>
       <x:c r="J23" s="1"/>
+      <x:c r="K23" s="1"/>
+      <x:c r="L23" s="1"/>
+      <x:c r="M23" s="1"/>
+      <x:c r="N23" s="1"/>
+      <x:c r="O23" s="1"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="1"/>
@@ -20382,6 +20660,11 @@
       <x:c r="H24" s="1"/>
       <x:c r="I24" s="1"/>
       <x:c r="J24" s="1"/>
+      <x:c r="K24" s="1"/>
+      <x:c r="L24" s="1"/>
+      <x:c r="M24" s="1"/>
+      <x:c r="N24" s="1"/>
+      <x:c r="O24" s="1"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="1"/>
@@ -20394,6 +20677,11 @@
       <x:c r="H25" s="1"/>
       <x:c r="I25" s="1"/>
       <x:c r="J25" s="1"/>
+      <x:c r="K25" s="1"/>
+      <x:c r="L25" s="1"/>
+      <x:c r="M25" s="1"/>
+      <x:c r="N25" s="1"/>
+      <x:c r="O25" s="1"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="1"/>
@@ -20406,6 +20694,11 @@
       <x:c r="H26" s="1"/>
       <x:c r="I26" s="1"/>
       <x:c r="J26" s="1"/>
+      <x:c r="K26" s="1"/>
+      <x:c r="L26" s="1"/>
+      <x:c r="M26" s="1"/>
+      <x:c r="N26" s="1"/>
+      <x:c r="O26" s="1"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="1"/>
@@ -20418,6 +20711,11 @@
       <x:c r="H27" s="1"/>
       <x:c r="I27" s="1"/>
       <x:c r="J27" s="1"/>
+      <x:c r="K27" s="1"/>
+      <x:c r="L27" s="1"/>
+      <x:c r="M27" s="1"/>
+      <x:c r="N27" s="1"/>
+      <x:c r="O27" s="1"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="1"/>
@@ -20430,6 +20728,11 @@
       <x:c r="H28" s="1"/>
       <x:c r="I28" s="1"/>
       <x:c r="J28" s="1"/>
+      <x:c r="K28" s="1"/>
+      <x:c r="L28" s="1"/>
+      <x:c r="M28" s="1"/>
+      <x:c r="N28" s="1"/>
+      <x:c r="O28" s="1"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="1"/>
@@ -20442,6 +20745,11 @@
       <x:c r="H29" s="1"/>
       <x:c r="I29" s="1"/>
       <x:c r="J29" s="1"/>
+      <x:c r="K29" s="1"/>
+      <x:c r="L29" s="1"/>
+      <x:c r="M29" s="1"/>
+      <x:c r="N29" s="1"/>
+      <x:c r="O29" s="1"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="1"/>
@@ -20454,6 +20762,11 @@
       <x:c r="H30" s="1"/>
       <x:c r="I30" s="1"/>
       <x:c r="J30" s="1"/>
+      <x:c r="K30" s="1"/>
+      <x:c r="L30" s="1"/>
+      <x:c r="M30" s="1"/>
+      <x:c r="N30" s="1"/>
+      <x:c r="O30" s="1"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="1"/>
@@ -20466,6 +20779,11 @@
       <x:c r="H31" s="1"/>
       <x:c r="I31" s="1"/>
       <x:c r="J31" s="1"/>
+      <x:c r="K31" s="1"/>
+      <x:c r="L31" s="1"/>
+      <x:c r="M31" s="1"/>
+      <x:c r="N31" s="1"/>
+      <x:c r="O31" s="1"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="1"/>
@@ -20478,6 +20796,11 @@
       <x:c r="H32" s="1"/>
       <x:c r="I32" s="1"/>
       <x:c r="J32" s="1"/>
+      <x:c r="K32" s="1"/>
+      <x:c r="L32" s="1"/>
+      <x:c r="M32" s="1"/>
+      <x:c r="N32" s="1"/>
+      <x:c r="O32" s="1"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="1"/>
@@ -20490,6 +20813,11 @@
       <x:c r="H33" s="1"/>
       <x:c r="I33" s="1"/>
       <x:c r="J33" s="1"/>
+      <x:c r="K33" s="1"/>
+      <x:c r="L33" s="1"/>
+      <x:c r="M33" s="1"/>
+      <x:c r="N33" s="1"/>
+      <x:c r="O33" s="1"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="1"/>
@@ -20502,6 +20830,11 @@
       <x:c r="H34" s="1"/>
       <x:c r="I34" s="1"/>
       <x:c r="J34" s="1"/>
+      <x:c r="K34" s="1"/>
+      <x:c r="L34" s="1"/>
+      <x:c r="M34" s="1"/>
+      <x:c r="N34" s="1"/>
+      <x:c r="O34" s="1"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="1"/>
@@ -20514,6 +20847,11 @@
       <x:c r="H35" s="1"/>
       <x:c r="I35" s="1"/>
       <x:c r="J35" s="1"/>
+      <x:c r="K35" s="1"/>
+      <x:c r="L35" s="1"/>
+      <x:c r="M35" s="1"/>
+      <x:c r="N35" s="1"/>
+      <x:c r="O35" s="1"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="1"/>
@@ -20526,6 +20864,11 @@
       <x:c r="H36" s="1"/>
       <x:c r="I36" s="1"/>
       <x:c r="J36" s="1"/>
+      <x:c r="K36" s="1"/>
+      <x:c r="L36" s="1"/>
+      <x:c r="M36" s="1"/>
+      <x:c r="N36" s="1"/>
+      <x:c r="O36" s="1"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="1"/>
@@ -20538,6 +20881,11 @@
       <x:c r="H37" s="1"/>
       <x:c r="I37" s="1"/>
       <x:c r="J37" s="1"/>
+      <x:c r="K37" s="1"/>
+      <x:c r="L37" s="1"/>
+      <x:c r="M37" s="1"/>
+      <x:c r="N37" s="1"/>
+      <x:c r="O37" s="1"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="1"/>
@@ -20550,6 +20898,11 @@
       <x:c r="H38" s="1"/>
       <x:c r="I38" s="1"/>
       <x:c r="J38" s="1"/>
+      <x:c r="K38" s="1"/>
+      <x:c r="L38" s="1"/>
+      <x:c r="M38" s="1"/>
+      <x:c r="N38" s="1"/>
+      <x:c r="O38" s="1"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="1"/>
@@ -20562,6 +20915,11 @@
       <x:c r="H39" s="1"/>
       <x:c r="I39" s="1"/>
       <x:c r="J39" s="1"/>
+      <x:c r="K39" s="1"/>
+      <x:c r="L39" s="1"/>
+      <x:c r="M39" s="1"/>
+      <x:c r="N39" s="1"/>
+      <x:c r="O39" s="1"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="1"/>
@@ -20574,6 +20932,11 @@
       <x:c r="H40" s="1"/>
       <x:c r="I40" s="1"/>
       <x:c r="J40" s="1"/>
+      <x:c r="K40" s="1"/>
+      <x:c r="L40" s="1"/>
+      <x:c r="M40" s="1"/>
+      <x:c r="N40" s="1"/>
+      <x:c r="O40" s="1"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="1"/>
@@ -20586,6 +20949,11 @@
       <x:c r="H41" s="1"/>
       <x:c r="I41" s="1"/>
       <x:c r="J41" s="1"/>
+      <x:c r="K41" s="1"/>
+      <x:c r="L41" s="1"/>
+      <x:c r="M41" s="1"/>
+      <x:c r="N41" s="1"/>
+      <x:c r="O41" s="1"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="1"/>
@@ -20598,6 +20966,11 @@
       <x:c r="H42" s="1"/>
       <x:c r="I42" s="1"/>
       <x:c r="J42" s="1"/>
+      <x:c r="K42" s="1"/>
+      <x:c r="L42" s="1"/>
+      <x:c r="M42" s="1"/>
+      <x:c r="N42" s="1"/>
+      <x:c r="O42" s="1"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="1"/>
@@ -20610,6 +20983,11 @@
       <x:c r="H43" s="1"/>
       <x:c r="I43" s="1"/>
       <x:c r="J43" s="1"/>
+      <x:c r="K43" s="1"/>
+      <x:c r="L43" s="1"/>
+      <x:c r="M43" s="1"/>
+      <x:c r="N43" s="1"/>
+      <x:c r="O43" s="1"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="1"/>
@@ -20622,6 +21000,11 @@
       <x:c r="H44" s="1"/>
       <x:c r="I44" s="1"/>
       <x:c r="J44" s="1"/>
+      <x:c r="K44" s="1"/>
+      <x:c r="L44" s="1"/>
+      <x:c r="M44" s="1"/>
+      <x:c r="N44" s="1"/>
+      <x:c r="O44" s="1"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="1"/>
@@ -20634,6 +21017,11 @@
       <x:c r="H45" s="1"/>
       <x:c r="I45" s="1"/>
       <x:c r="J45" s="1"/>
+      <x:c r="K45" s="1"/>
+      <x:c r="L45" s="1"/>
+      <x:c r="M45" s="1"/>
+      <x:c r="N45" s="1"/>
+      <x:c r="O45" s="1"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="1"/>
@@ -20646,6 +21034,11 @@
       <x:c r="H46" s="1"/>
       <x:c r="I46" s="1"/>
       <x:c r="J46" s="1"/>
+      <x:c r="K46" s="1"/>
+      <x:c r="L46" s="1"/>
+      <x:c r="M46" s="1"/>
+      <x:c r="N46" s="1"/>
+      <x:c r="O46" s="1"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="1"/>
@@ -20658,6 +21051,11 @@
       <x:c r="H47" s="1"/>
       <x:c r="I47" s="1"/>
       <x:c r="J47" s="1"/>
+      <x:c r="K47" s="1"/>
+      <x:c r="L47" s="1"/>
+      <x:c r="M47" s="1"/>
+      <x:c r="N47" s="1"/>
+      <x:c r="O47" s="1"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="1"/>
@@ -20670,6 +21068,11 @@
       <x:c r="H48" s="1"/>
       <x:c r="I48" s="1"/>
       <x:c r="J48" s="1"/>
+      <x:c r="K48" s="1"/>
+      <x:c r="L48" s="1"/>
+      <x:c r="M48" s="1"/>
+      <x:c r="N48" s="1"/>
+      <x:c r="O48" s="1"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="1"/>
@@ -20682,6 +21085,11 @@
       <x:c r="H49" s="1"/>
       <x:c r="I49" s="1"/>
       <x:c r="J49" s="1"/>
+      <x:c r="K49" s="1"/>
+      <x:c r="L49" s="1"/>
+      <x:c r="M49" s="1"/>
+      <x:c r="N49" s="1"/>
+      <x:c r="O49" s="1"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="1"/>
@@ -20694,6 +21102,11 @@
       <x:c r="H50" s="1"/>
       <x:c r="I50" s="1"/>
       <x:c r="J50" s="1"/>
+      <x:c r="K50" s="1"/>
+      <x:c r="L50" s="1"/>
+      <x:c r="M50" s="1"/>
+      <x:c r="N50" s="1"/>
+      <x:c r="O50" s="1"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="1"/>
@@ -20706,6 +21119,11 @@
       <x:c r="H51" s="1"/>
       <x:c r="I51" s="1"/>
       <x:c r="J51" s="1"/>
+      <x:c r="K51" s="1"/>
+      <x:c r="L51" s="1"/>
+      <x:c r="M51" s="1"/>
+      <x:c r="N51" s="1"/>
+      <x:c r="O51" s="1"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="1"/>
@@ -20718,6 +21136,11 @@
       <x:c r="H52" s="1"/>
       <x:c r="I52" s="1"/>
       <x:c r="J52" s="1"/>
+      <x:c r="K52" s="1"/>
+      <x:c r="L52" s="1"/>
+      <x:c r="M52" s="1"/>
+      <x:c r="N52" s="1"/>
+      <x:c r="O52" s="1"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="1"/>
@@ -20730,6 +21153,11 @@
       <x:c r="H53" s="1"/>
       <x:c r="I53" s="1"/>
       <x:c r="J53" s="1"/>
+      <x:c r="K53" s="1"/>
+      <x:c r="L53" s="1"/>
+      <x:c r="M53" s="1"/>
+      <x:c r="N53" s="1"/>
+      <x:c r="O53" s="1"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="1"/>
@@ -20742,6 +21170,11 @@
       <x:c r="H54" s="1"/>
       <x:c r="I54" s="1"/>
       <x:c r="J54" s="1"/>
+      <x:c r="K54" s="1"/>
+      <x:c r="L54" s="1"/>
+      <x:c r="M54" s="1"/>
+      <x:c r="N54" s="1"/>
+      <x:c r="O54" s="1"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="1"/>
@@ -20754,6 +21187,11 @@
       <x:c r="H55" s="1"/>
       <x:c r="I55" s="1"/>
       <x:c r="J55" s="1"/>
+      <x:c r="K55" s="1"/>
+      <x:c r="L55" s="1"/>
+      <x:c r="M55" s="1"/>
+      <x:c r="N55" s="1"/>
+      <x:c r="O55" s="1"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="1"/>
@@ -20766,6 +21204,11 @@
       <x:c r="H56" s="1"/>
       <x:c r="I56" s="1"/>
       <x:c r="J56" s="1"/>
+      <x:c r="K56" s="1"/>
+      <x:c r="L56" s="1"/>
+      <x:c r="M56" s="1"/>
+      <x:c r="N56" s="1"/>
+      <x:c r="O56" s="1"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="1"/>
@@ -20778,6 +21221,11 @@
       <x:c r="H57" s="1"/>
       <x:c r="I57" s="1"/>
       <x:c r="J57" s="1"/>
+      <x:c r="K57" s="1"/>
+      <x:c r="L57" s="1"/>
+      <x:c r="M57" s="1"/>
+      <x:c r="N57" s="1"/>
+      <x:c r="O57" s="1"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="1"/>
@@ -20790,6 +21238,11 @@
       <x:c r="H58" s="1"/>
       <x:c r="I58" s="1"/>
       <x:c r="J58" s="1"/>
+      <x:c r="K58" s="1"/>
+      <x:c r="L58" s="1"/>
+      <x:c r="M58" s="1"/>
+      <x:c r="N58" s="1"/>
+      <x:c r="O58" s="1"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="1"/>
@@ -20802,6 +21255,11 @@
       <x:c r="H59" s="1"/>
       <x:c r="I59" s="1"/>
       <x:c r="J59" s="1"/>
+      <x:c r="K59" s="1"/>
+      <x:c r="L59" s="1"/>
+      <x:c r="M59" s="1"/>
+      <x:c r="N59" s="1"/>
+      <x:c r="O59" s="1"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="1"/>
@@ -20814,6 +21272,11 @@
       <x:c r="H60" s="1"/>
       <x:c r="I60" s="1"/>
       <x:c r="J60" s="1"/>
+      <x:c r="K60" s="1"/>
+      <x:c r="L60" s="1"/>
+      <x:c r="M60" s="1"/>
+      <x:c r="N60" s="1"/>
+      <x:c r="O60" s="1"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="1"/>
@@ -20826,6 +21289,11 @@
       <x:c r="H61" s="1"/>
       <x:c r="I61" s="1"/>
       <x:c r="J61" s="1"/>
+      <x:c r="K61" s="1"/>
+      <x:c r="L61" s="1"/>
+      <x:c r="M61" s="1"/>
+      <x:c r="N61" s="1"/>
+      <x:c r="O61" s="1"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="1"/>
@@ -20838,6 +21306,11 @@
       <x:c r="H62" s="1"/>
       <x:c r="I62" s="1"/>
       <x:c r="J62" s="1"/>
+      <x:c r="K62" s="1"/>
+      <x:c r="L62" s="1"/>
+      <x:c r="M62" s="1"/>
+      <x:c r="N62" s="1"/>
+      <x:c r="O62" s="1"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="1"/>
@@ -20850,6 +21323,11 @@
       <x:c r="H63" s="1"/>
       <x:c r="I63" s="1"/>
       <x:c r="J63" s="1"/>
+      <x:c r="K63" s="1"/>
+      <x:c r="L63" s="1"/>
+      <x:c r="M63" s="1"/>
+      <x:c r="N63" s="1"/>
+      <x:c r="O63" s="1"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="1"/>
@@ -20862,6 +21340,11 @@
       <x:c r="H64" s="1"/>
       <x:c r="I64" s="1"/>
       <x:c r="J64" s="1"/>
+      <x:c r="K64" s="1"/>
+      <x:c r="L64" s="1"/>
+      <x:c r="M64" s="1"/>
+      <x:c r="N64" s="1"/>
+      <x:c r="O64" s="1"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="1"/>
@@ -20874,6 +21357,11 @@
       <x:c r="H65" s="1"/>
       <x:c r="I65" s="1"/>
       <x:c r="J65" s="1"/>
+      <x:c r="K65" s="1"/>
+      <x:c r="L65" s="1"/>
+      <x:c r="M65" s="1"/>
+      <x:c r="N65" s="1"/>
+      <x:c r="O65" s="1"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="1"/>
@@ -20886,6 +21374,11 @@
       <x:c r="H66" s="1"/>
       <x:c r="I66" s="1"/>
       <x:c r="J66" s="1"/>
+      <x:c r="K66" s="1"/>
+      <x:c r="L66" s="1"/>
+      <x:c r="M66" s="1"/>
+      <x:c r="N66" s="1"/>
+      <x:c r="O66" s="1"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="1"/>
@@ -20898,6 +21391,11 @@
       <x:c r="H67" s="1"/>
       <x:c r="I67" s="1"/>
       <x:c r="J67" s="1"/>
+      <x:c r="K67" s="1"/>
+      <x:c r="L67" s="1"/>
+      <x:c r="M67" s="1"/>
+      <x:c r="N67" s="1"/>
+      <x:c r="O67" s="1"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="1"/>
@@ -20910,6 +21408,11 @@
       <x:c r="H68" s="1"/>
       <x:c r="I68" s="1"/>
       <x:c r="J68" s="1"/>
+      <x:c r="K68" s="1"/>
+      <x:c r="L68" s="1"/>
+      <x:c r="M68" s="1"/>
+      <x:c r="N68" s="1"/>
+      <x:c r="O68" s="1"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="1"/>
@@ -20922,6 +21425,11 @@
       <x:c r="H69" s="1"/>
       <x:c r="I69" s="1"/>
       <x:c r="J69" s="1"/>
+      <x:c r="K69" s="1"/>
+      <x:c r="L69" s="1"/>
+      <x:c r="M69" s="1"/>
+      <x:c r="N69" s="1"/>
+      <x:c r="O69" s="1"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="1"/>
@@ -20934,6 +21442,11 @@
       <x:c r="H70" s="1"/>
       <x:c r="I70" s="1"/>
       <x:c r="J70" s="1"/>
+      <x:c r="K70" s="1"/>
+      <x:c r="L70" s="1"/>
+      <x:c r="M70" s="1"/>
+      <x:c r="N70" s="1"/>
+      <x:c r="O70" s="1"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="1"/>
@@ -20946,6 +21459,11 @@
       <x:c r="H71" s="1"/>
       <x:c r="I71" s="1"/>
       <x:c r="J71" s="1"/>
+      <x:c r="K71" s="1"/>
+      <x:c r="L71" s="1"/>
+      <x:c r="M71" s="1"/>
+      <x:c r="N71" s="1"/>
+      <x:c r="O71" s="1"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="1"/>
@@ -20958,6 +21476,11 @@
       <x:c r="H72" s="1"/>
       <x:c r="I72" s="1"/>
       <x:c r="J72" s="1"/>
+      <x:c r="K72" s="1"/>
+      <x:c r="L72" s="1"/>
+      <x:c r="M72" s="1"/>
+      <x:c r="N72" s="1"/>
+      <x:c r="O72" s="1"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="1"/>
@@ -20970,6 +21493,11 @@
       <x:c r="H73" s="1"/>
       <x:c r="I73" s="1"/>
       <x:c r="J73" s="1"/>
+      <x:c r="K73" s="1"/>
+      <x:c r="L73" s="1"/>
+      <x:c r="M73" s="1"/>
+      <x:c r="N73" s="1"/>
+      <x:c r="O73" s="1"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="1"/>
@@ -20982,6 +21510,11 @@
       <x:c r="H74" s="1"/>
       <x:c r="I74" s="1"/>
       <x:c r="J74" s="1"/>
+      <x:c r="K74" s="1"/>
+      <x:c r="L74" s="1"/>
+      <x:c r="M74" s="1"/>
+      <x:c r="N74" s="1"/>
+      <x:c r="O74" s="1"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="1"/>
@@ -20994,6 +21527,11 @@
       <x:c r="H75" s="1"/>
       <x:c r="I75" s="1"/>
       <x:c r="J75" s="1"/>
+      <x:c r="K75" s="1"/>
+      <x:c r="L75" s="1"/>
+      <x:c r="M75" s="1"/>
+      <x:c r="N75" s="1"/>
+      <x:c r="O75" s="1"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="1"/>
@@ -21006,6 +21544,11 @@
       <x:c r="H76" s="1"/>
       <x:c r="I76" s="1"/>
       <x:c r="J76" s="1"/>
+      <x:c r="K76" s="1"/>
+      <x:c r="L76" s="1"/>
+      <x:c r="M76" s="1"/>
+      <x:c r="N76" s="1"/>
+      <x:c r="O76" s="1"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="1"/>
@@ -21018,6 +21561,11 @@
       <x:c r="H77" s="1"/>
       <x:c r="I77" s="1"/>
       <x:c r="J77" s="1"/>
+      <x:c r="K77" s="1"/>
+      <x:c r="L77" s="1"/>
+      <x:c r="M77" s="1"/>
+      <x:c r="N77" s="1"/>
+      <x:c r="O77" s="1"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="1"/>
@@ -21030,6 +21578,11 @@
       <x:c r="H78" s="1"/>
       <x:c r="I78" s="1"/>
       <x:c r="J78" s="1"/>
+      <x:c r="K78" s="1"/>
+      <x:c r="L78" s="1"/>
+      <x:c r="M78" s="1"/>
+      <x:c r="N78" s="1"/>
+      <x:c r="O78" s="1"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="1"/>
@@ -21042,6 +21595,11 @@
       <x:c r="H79" s="1"/>
       <x:c r="I79" s="1"/>
       <x:c r="J79" s="1"/>
+      <x:c r="K79" s="1"/>
+      <x:c r="L79" s="1"/>
+      <x:c r="M79" s="1"/>
+      <x:c r="N79" s="1"/>
+      <x:c r="O79" s="1"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="1"/>
@@ -21054,16 +21612,25 @@
       <x:c r="H80" s="1"/>
       <x:c r="I80" s="1"/>
       <x:c r="J80" s="1"/>
+      <x:c r="K80" s="1"/>
+      <x:c r="L80" s="1"/>
+      <x:c r="M80" s="1"/>
+      <x:c r="N80" s="1"/>
+      <x:c r="O80" s="1"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:J1"/>
-    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L2"/>
     <x:mergeCell ref="A4:B4"/>
     <x:mergeCell ref="E4:F4"/>
+    <x:mergeCell ref="I4:J4"/>
+    <x:mergeCell ref="K4:L4"/>
+    <x:mergeCell ref="I5:J5"/>
+    <x:mergeCell ref="K5:L5"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00d66583a23d448d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21b4aebcef4941b2"/>
 </x:worksheet>
 </file>
 
@@ -21200,7 +21767,7 @@
         <x:f>B8+C8</x:f>
         <x:v>-1500</x:v>
       </x:c>
-      <x:c r="E8" s="69" t="n">
+      <x:c r="E8" s="87" t="n">
         <x:f>ABS(D8)/Assumptions!$B$10</x:f>
         <x:v>0.06666666666666667</x:v>
       </x:c>
@@ -21235,7 +21802,7 @@
         <x:f>B9+C9</x:f>
         <x:v>-6000</x:v>
       </x:c>
-      <x:c r="E9" s="69" t="n">
+      <x:c r="E9" s="87" t="n">
         <x:f>ABS(D9)/Assumptions!$B$10</x:f>
         <x:v>0.26666666666666666</x:v>
       </x:c>
@@ -21332,147 +21899,147 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="32" customHeight="1">
-      <x:c r="A15" s="70" t="str">
+      <x:c r="A15" s="88" t="str">
         <x:v>IRRBB_DV01</x:v>
       </x:c>
-      <x:c r="B15" s="70" t="str">
+      <x:c r="B15" s="88" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="C15" s="70" t="str">
+      <x:c r="C15" s="88" t="str">
         <x:v>plain_vanilla_interest_rate_swap</x:v>
       </x:c>
-      <x:c r="D15" s="70" t="str">
+      <x:c r="D15" s="88" t="str">
         <x:v>PAY_FIXED_RECEIVE_FLOAT</x:v>
       </x:c>
-      <x:c r="E15" s="71" t="n">
+      <x:c r="E15" s="89" t="n">
         <x:v>438.50875</x:v>
       </x:c>
-      <x:c r="F15" s="71" t="n">
+      <x:c r="F15" s="89" t="n">
         <x:v>-0.350807</x:v>
       </x:c>
-      <x:c r="G15" s="71" t="n">
+      <x:c r="G15" s="89" t="n">
         <x:v>-0.175404</x:v>
       </x:c>
-      <x:c r="H15" s="71" t="n">
+      <x:c r="H15" s="89" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="I15" s="72" t="str">
+      <x:c r="I15" s="90" t="str">
         <x:v>ALCO_REVIEW_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="32" customHeight="1">
-      <x:c r="A16" s="70" t="str">
+      <x:c r="A16" s="88" t="str">
         <x:v>IRRBB_DV01</x:v>
       </x:c>
-      <x:c r="B16" s="70" t="str">
+      <x:c r="B16" s="88" t="str">
         <x:v>TRY</x:v>
       </x:c>
-      <x:c r="C16" s="70" t="str">
+      <x:c r="C16" s="88" t="str">
         <x:v>plain_vanilla_interest_rate_swap</x:v>
       </x:c>
-      <x:c r="D16" s="70" t="str">
+      <x:c r="D16" s="88" t="str">
         <x:v>PAY_FIXED_RECEIVE_FLOAT</x:v>
       </x:c>
-      <x:c r="E16" s="71" t="n">
+      <x:c r="E16" s="89" t="n">
         <x:v>10316.64625</x:v>
       </x:c>
-      <x:c r="F16" s="71" t="n">
+      <x:c r="F16" s="89" t="n">
         <x:v>-8.253317</x:v>
       </x:c>
-      <x:c r="G16" s="71" t="n">
+      <x:c r="G16" s="89" t="n">
         <x:v>-4.126658</x:v>
       </x:c>
-      <x:c r="H16" s="71" t="n">
+      <x:c r="H16" s="89" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="I16" s="72" t="str">
+      <x:c r="I16" s="90" t="str">
         <x:v>ALCO_REVIEW_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="32" customHeight="1">
-      <x:c r="A17" s="70" t="str">
+      <x:c r="A17" s="88" t="str">
         <x:v>IRRBB_DV01</x:v>
       </x:c>
-      <x:c r="B17" s="70" t="str">
+      <x:c r="B17" s="88" t="str">
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="C17" s="70" t="str">
+      <x:c r="C17" s="88" t="str">
         <x:v>plain_vanilla_interest_rate_swap</x:v>
       </x:c>
-      <x:c r="D17" s="70" t="str">
+      <x:c r="D17" s="88" t="str">
         <x:v>RECEIVE_FIXED_PAY_FLOAT</x:v>
       </x:c>
-      <x:c r="E17" s="71" t="n">
+      <x:c r="E17" s="89" t="n">
         <x:v>163.53</x:v>
       </x:c>
-      <x:c r="F17" s="71" t="n">
+      <x:c r="F17" s="89" t="n">
         <x:v>0.130824</x:v>
       </x:c>
-      <x:c r="G17" s="71" t="n">
+      <x:c r="G17" s="89" t="n">
         <x:v>0.065412</x:v>
       </x:c>
-      <x:c r="H17" s="71" t="n">
+      <x:c r="H17" s="89" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="I17" s="72" t="str">
+      <x:c r="I17" s="90" t="str">
         <x:v>ALCO_REVIEW_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="32" customHeight="1">
-      <x:c r="A18" s="70" t="str">
+      <x:c r="A18" s="88" t="str">
         <x:v>FX_OPEN_POSITION</x:v>
       </x:c>
-      <x:c r="B18" s="70" t="str">
+      <x:c r="B18" s="88" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="C18" s="70" t="str">
+      <x:c r="C18" s="88" t="str">
         <x:v>fx_swap_or_forward</x:v>
       </x:c>
-      <x:c r="D18" s="70" t="str">
+      <x:c r="D18" s="88" t="str">
         <x:v>BUY_FX_SELL_TRY</x:v>
       </x:c>
-      <x:c r="E18" s="71" t="n">
+      <x:c r="E18" s="89" t="n">
         <x:v>1200</x:v>
       </x:c>
-      <x:c r="F18" s="71" t="n">
+      <x:c r="F18" s="89" t="n">
         <x:v>-1500</x:v>
       </x:c>
-      <x:c r="G18" s="71" t="n">
+      <x:c r="G18" s="89" t="n">
         <x:v>-300</x:v>
       </x:c>
-      <x:c r="H18" s="71" t="n">
+      <x:c r="H18" s="89" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="I18" s="72" t="str">
+      <x:c r="I18" s="90" t="str">
         <x:v>ALCO_REVIEW_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="32" customHeight="1">
-      <x:c r="A19" s="70" t="str">
+      <x:c r="A19" s="88" t="str">
         <x:v>FX_OPEN_POSITION</x:v>
       </x:c>
-      <x:c r="B19" s="70" t="str">
+      <x:c r="B19" s="88" t="str">
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="C19" s="70" t="str">
+      <x:c r="C19" s="88" t="str">
         <x:v>fx_swap_or_forward</x:v>
       </x:c>
-      <x:c r="D19" s="70" t="str">
+      <x:c r="D19" s="88" t="str">
         <x:v>BUY_FX_SELL_TRY</x:v>
       </x:c>
-      <x:c r="E19" s="71" t="n">
+      <x:c r="E19" s="89" t="n">
         <x:v>4800</x:v>
       </x:c>
-      <x:c r="F19" s="71" t="n">
+      <x:c r="F19" s="89" t="n">
         <x:v>-6000</x:v>
       </x:c>
-      <x:c r="G19" s="71" t="n">
+      <x:c r="G19" s="89" t="n">
         <x:v>-1200</x:v>
       </x:c>
-      <x:c r="H19" s="71" t="n">
+      <x:c r="H19" s="89" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="I19" s="72" t="str">
+      <x:c r="I19" s="90" t="str">
         <x:v>ALCO_REVIEW_REQUIRED</x:v>
       </x:c>
     </x:row>

</xml_diff>